<commit_message>
Add Scored+Actions worksheet to The Cove LEED-ND scorecard
New front sheet 'The Cove - Scored + Actions': every prerequisite and credit
scored as-is (Now), achievable ceiling (Potential), color-coded Status, and a
concrete 'what to do to bring it up to speed' action per line. Interpretive
total: 20 now / 38 potential of 110 (below the 40-pt Certified floor), with
structural rezoning + green-building notes for the path to Certified/Silver.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C83XSMHt5roS8jvvJWFf8j
</commit_message>
<xml_diff>
--- a/the_cove_deerfield_beach/the_cove_LEED_ND_scorecard.xlsx
+++ b/the_cove_deerfield_beach/the_cove_LEED_ND_scorecard.xlsx
@@ -6,12 +6,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="90" yWindow="450" windowWidth="12390" windowHeight="5085" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Neighborhood Development Plan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Neighborhood Development" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="The Cove - Scored + Actions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Neighborhood Development Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Neighborhood Development" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Neighborhood Development Plan'!$A$1:$Q$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Neighborhood Development'!$A$1:$Q$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Neighborhood Development Plan'!$A$1:$Q$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Neighborhood Development'!$A$1:$Q$42</definedName>
   </definedNames>
   <calcPr calcId="145621" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -185,8 +186,33 @@
       <color indexed="63"/>
       <sz val="8"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E5F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -229,8 +255,43 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDE7EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -355,11 +416,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -693,6 +768,56 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="11" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -994,6 +1119,1998 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G75"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="72" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="100" t="inlineStr">
+        <is>
+          <t>The Cove, Deerfield Beach FL - LEED-ND Scored As-Is + Actions to Improve</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="101" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B2" s="101" t="inlineStr">
+        <is>
+          <t>Credit / Prerequisite</t>
+        </is>
+      </c>
+      <c r="C2" s="102" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="D2" s="102" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="E2" s="102" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="F2" s="102" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G2" s="101" t="inlineStr">
+        <is>
+          <t>What to do to bring it up to speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="103" t="inlineStr">
+        <is>
+          <t>SMART LOCATION &amp; LINKAGE (max 28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B4" s="105" t="inlineStr">
+        <is>
+          <t>Smart Location</t>
+        </is>
+      </c>
+      <c r="C4" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D4" s="106" t="inlineStr"/>
+      <c r="E4" s="106" t="inlineStr"/>
+      <c r="F4" s="107" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="G4" s="105" t="inlineStr">
+        <is>
+          <t>Infill site already qualifies. Maintain; document adjacency/connectivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B5" s="105" t="inlineStr">
+        <is>
+          <t>Imperiled Species &amp; Ecological Communities</t>
+        </is>
+      </c>
+      <c r="C5" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D5" s="106" t="inlineStr"/>
+      <c r="E5" s="106" t="inlineStr"/>
+      <c r="F5" s="108" t="inlineStr">
+        <is>
+          <t>Met (verify)</t>
+        </is>
+      </c>
+      <c r="G5" s="105" t="inlineStr">
+        <is>
+          <t>Pull FWC/USFWS records to confirm no listed-species habitat; keep documentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B6" s="105" t="inlineStr">
+        <is>
+          <t>Wetland &amp; Water Body Conservation</t>
+        </is>
+      </c>
+      <c r="C6" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D6" s="106" t="inlineStr"/>
+      <c r="E6" s="106" t="inlineStr"/>
+      <c r="F6" s="109" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="G6" s="105" t="inlineStr">
+        <is>
+          <t>Built to seawalls, no buffers. Add living shorelines / vegetated canal buffers where feasible; document existing condition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B7" s="105" t="inlineStr">
+        <is>
+          <t>Agricultural Land Conservation</t>
+        </is>
+      </c>
+      <c r="C7" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D7" s="106" t="inlineStr"/>
+      <c r="E7" s="106" t="inlineStr"/>
+      <c r="F7" s="108" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" s="105" t="inlineStr">
+        <is>
+          <t>No farmland - no action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B8" s="105" t="inlineStr">
+        <is>
+          <t>Floodplain Avoidance</t>
+        </is>
+      </c>
+      <c r="C8" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D8" s="106" t="inlineStr"/>
+      <c r="E8" s="106" t="inlineStr"/>
+      <c r="F8" s="109" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="G8" s="105" t="inlineStr">
+        <is>
+          <t>Largely FEMA Zone AE. Qualify via the previously-developed/infill path; adopt freeboard + flood-resilient construction standards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B9" s="105" t="inlineStr">
+        <is>
+          <t>Preferred Locations</t>
+        </is>
+      </c>
+      <c r="C9" s="106" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="106" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="106" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G9" s="105" t="inlineStr">
+        <is>
+          <t>Document intersection density &amp; adjacency; add east-side street/ped connections to raise the score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B10" s="105" t="inlineStr">
+        <is>
+          <t>Brownfield Remediation</t>
+        </is>
+      </c>
+      <c r="C10" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="108" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G10" s="105" t="inlineStr">
+        <is>
+          <t>No known brownfield; only pursue if a contaminated parcel is identified &amp; cleaned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B11" s="105" t="inlineStr">
+        <is>
+          <t>Access to Quality Transit</t>
+        </is>
+      </c>
+      <c r="C11" s="106" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="106" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G11" s="105" t="inlineStr">
+        <is>
+          <t>Partner with Broward County Transit for higher bus frequency on US-1/Hillsboro; add sheltered stops; document service levels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B12" s="105" t="inlineStr">
+        <is>
+          <t>Bicycle Facilities</t>
+        </is>
+      </c>
+      <c r="C12" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G12" s="105" t="inlineStr">
+        <is>
+          <t>Add bike lanes + racks linking the Cove node, beach and A1A; connect to the county bike network.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B13" s="105" t="inlineStr">
+        <is>
+          <t>Housing and Jobs Proximity</t>
+        </is>
+      </c>
+      <c r="C13" s="106" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G13" s="105" t="inlineStr">
+        <is>
+          <t>Document jobs within 1/2 mile (Cove retail + Hillsboro corridor); add jobs through mixed-use edge redevelopment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B14" s="105" t="inlineStr">
+        <is>
+          <t>Steep Slope Protection</t>
+        </is>
+      </c>
+      <c r="C14" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="108" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G14" s="105" t="inlineStr">
+        <is>
+          <t>Flat coastal site - not achievable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B15" s="105" t="inlineStr">
+        <is>
+          <t>Site Design for Habitat/Water Body</t>
+        </is>
+      </c>
+      <c r="C15" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G15" s="105" t="inlineStr">
+        <is>
+          <t>Add native shoreline planting / habitat features along canals &amp; the ICW to pursue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B16" s="105" t="inlineStr">
+        <is>
+          <t>Restoration of Habitat/Wetlands</t>
+        </is>
+      </c>
+      <c r="C16" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G16" s="105" t="inlineStr">
+        <is>
+          <t>Restore a mangrove/native edge segment (e.g., near Sullivan Park) to earn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B17" s="105" t="inlineStr">
+        <is>
+          <t>Long-Term Conservation Management</t>
+        </is>
+      </c>
+      <c r="C17" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G17" s="105" t="inlineStr">
+        <is>
+          <t>Adopt a written long-term management plan for any restored habitat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="111" t="n"/>
+      <c r="B18" s="112" t="inlineStr">
+        <is>
+          <t>Subtotal - Smart Location &amp; Linkage</t>
+        </is>
+      </c>
+      <c r="C18" s="102" t="n">
+        <v>28</v>
+      </c>
+      <c r="D18" s="102" t="n">
+        <v>7</v>
+      </c>
+      <c r="E18" s="102" t="n">
+        <v>13</v>
+      </c>
+      <c r="F18" s="111" t="n"/>
+      <c r="G18" s="111" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="103" t="inlineStr">
+        <is>
+          <t>NEIGHBORHOOD PATTERN &amp; DESIGN (max 41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B20" s="105" t="inlineStr">
+        <is>
+          <t>Walkable Streets</t>
+        </is>
+      </c>
+      <c r="C20" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D20" s="106" t="inlineStr"/>
+      <c r="E20" s="106" t="inlineStr"/>
+      <c r="F20" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G20" s="105" t="inlineStr">
+        <is>
+          <t>Sidewalk-gap audit; fill missing segments; require building entries to face the street on corridors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B21" s="105" t="inlineStr">
+        <is>
+          <t>Compact Development</t>
+        </is>
+      </c>
+      <c r="C21" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D21" s="106" t="inlineStr"/>
+      <c r="E21" s="106" t="inlineStr"/>
+      <c r="F21" s="109" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="G21" s="105" t="inlineStr">
+        <is>
+          <t>Single-family density is below the minimum. Raise allowed net density on US-1 &amp; Hillsboro edges to satisfy the prereq.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B22" s="105" t="inlineStr">
+        <is>
+          <t>Connected &amp; Open Community</t>
+        </is>
+      </c>
+      <c r="C22" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D22" s="106" t="inlineStr"/>
+      <c r="E22" s="106" t="inlineStr"/>
+      <c r="F22" s="109" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="G22" s="105" t="inlineStr">
+        <is>
+          <t>Improve intersection density; add pedestrian cut-throughs between finger-canal streets; keep streets public.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B23" s="105" t="inlineStr">
+        <is>
+          <t>Walkable Streets</t>
+        </is>
+      </c>
+      <c r="C23" s="106" t="n">
+        <v>9</v>
+      </c>
+      <c r="D23" s="106" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" s="106" t="n">
+        <v>5</v>
+      </c>
+      <c r="F23" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G23" s="105" t="inlineStr">
+        <is>
+          <t>Continuous sidewalks, street trees, on-street parking, and facade/entry standards along US-1 &amp; Hillsboro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B24" s="105" t="inlineStr">
+        <is>
+          <t>Compact Development</t>
+        </is>
+      </c>
+      <c r="C24" s="106" t="n">
+        <v>6</v>
+      </c>
+      <c r="D24" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="109" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="G24" s="105" t="inlineStr">
+        <is>
+          <t>Allow mixed-use / multifamily infill on the two arterial edges to lift net residential density.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B25" s="105" t="inlineStr">
+        <is>
+          <t>Mixed-Use Neighborhoods</t>
+        </is>
+      </c>
+      <c r="C25" s="106" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G25" s="105" t="inlineStr">
+        <is>
+          <t>Encourage ground-floor retail + housing at the Cove node and along US-1; broaden the use mix within walking distance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B26" s="105" t="inlineStr">
+        <is>
+          <t>Housing Types and Affordability</t>
+        </is>
+      </c>
+      <c r="C26" s="106" t="n">
+        <v>7</v>
+      </c>
+      <c r="D26" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="109" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="G26" s="105" t="inlineStr">
+        <is>
+          <t>Add housing types (townhome/duplex/ADU/apartment) and income-restricted units on corridor infill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B27" s="105" t="inlineStr">
+        <is>
+          <t>Reduced Parking Footprint</t>
+        </is>
+      </c>
+      <c r="C27" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G27" s="105" t="inlineStr">
+        <is>
+          <t>Shared/structured parking + reduced minimums at the shopping center; convert some surface lot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B28" s="105" t="inlineStr">
+        <is>
+          <t>Connected and Open Community</t>
+        </is>
+      </c>
+      <c r="C28" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G28" s="105" t="inlineStr">
+        <is>
+          <t>Add ped/bike connections; ensure new streets are public and through-connected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B29" s="105" t="inlineStr">
+        <is>
+          <t>Transit Facilities</t>
+        </is>
+      </c>
+      <c r="C29" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="107" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="G29" s="105" t="inlineStr">
+        <is>
+          <t>Maintain shelters/benches at stops; add real-time arrival info.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B30" s="105" t="inlineStr">
+        <is>
+          <t>Transportation Demand Management</t>
+        </is>
+      </c>
+      <c r="C30" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G30" s="105" t="inlineStr">
+        <is>
+          <t>Launch a TDM program (transit passes, bike share, carpool) anchored at the retail node.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B31" s="105" t="inlineStr">
+        <is>
+          <t>Access to Civic &amp; Public Space</t>
+        </is>
+      </c>
+      <c r="C31" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="107" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="G31" s="105" t="inlineStr">
+        <is>
+          <t>Maintain Sullivan Park promenade and public waterfront access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B32" s="105" t="inlineStr">
+        <is>
+          <t>Access to Recreation Facilities</t>
+        </is>
+      </c>
+      <c r="C32" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="107" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="G32" s="105" t="inlineStr">
+        <is>
+          <t>Maintain access to parks, pier, beach and Deerfield Island Park.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B33" s="105" t="inlineStr">
+        <is>
+          <t>Visitability and Universal Design</t>
+        </is>
+      </c>
+      <c r="C33" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G33" s="105" t="inlineStr">
+        <is>
+          <t>Adopt visitability standards (zero-step entry, wider doors) for new/renovated homes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B34" s="105" t="inlineStr">
+        <is>
+          <t>Community Outreach and Involvement</t>
+        </is>
+      </c>
+      <c r="C34" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G34" s="105" t="inlineStr">
+        <is>
+          <t>Formalize a charrette/engagement process with the Cove Civic Association and document it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B35" s="105" t="inlineStr">
+        <is>
+          <t>Local Food Production</t>
+        </is>
+      </c>
+      <c r="C35" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="107" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="G35" s="105" t="inlineStr">
+        <is>
+          <t>Sustain the farmers market; add community-garden space.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B36" s="105" t="inlineStr">
+        <is>
+          <t>Tree-Lined and Shaded Streetscapes</t>
+        </is>
+      </c>
+      <c r="C36" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="F36" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G36" s="105" t="inlineStr">
+        <is>
+          <t>Canopy inventory + street-tree planting program to meet the shading thresholds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B37" s="105" t="inlineStr">
+        <is>
+          <t>Neighborhood Schools</t>
+        </is>
+      </c>
+      <c r="C37" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="107" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="G37" s="105" t="inlineStr">
+        <is>
+          <t>Maintain walkable access to St. Ambrose / Deerfield schools; add safe-routes-to-school.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="111" t="n"/>
+      <c r="B38" s="112" t="inlineStr">
+        <is>
+          <t>Subtotal - Neighborhood Pattern &amp; Design</t>
+        </is>
+      </c>
+      <c r="C38" s="102" t="n">
+        <v>41</v>
+      </c>
+      <c r="D38" s="102" t="n">
+        <v>11</v>
+      </c>
+      <c r="E38" s="102" t="n">
+        <v>19</v>
+      </c>
+      <c r="F38" s="111" t="n"/>
+      <c r="G38" s="111" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="103" t="inlineStr">
+        <is>
+          <t>GREEN INFRASTRUCTURE &amp; BUILDINGS (max 31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B40" s="105" t="inlineStr">
+        <is>
+          <t>Certified Green Building</t>
+        </is>
+      </c>
+      <c r="C40" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D40" s="106" t="inlineStr"/>
+      <c r="E40" s="106" t="inlineStr"/>
+      <c r="F40" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G40" s="105" t="inlineStr">
+        <is>
+          <t>DECISIVE GAP. Require &gt;=1 green-certified building (LEED/FGBC) in any new construction or major renovation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B41" s="105" t="inlineStr">
+        <is>
+          <t>Minimum Building Energy Performance</t>
+        </is>
+      </c>
+      <c r="C41" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D41" s="106" t="inlineStr"/>
+      <c r="E41" s="106" t="inlineStr"/>
+      <c r="F41" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G41" s="105" t="inlineStr">
+        <is>
+          <t>Existing 1956 stock. Require energy-code compliance + retrofit incentives; document on new/renovated buildings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B42" s="105" t="inlineStr">
+        <is>
+          <t>Indoor Water Use Reduction</t>
+        </is>
+      </c>
+      <c r="C42" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D42" s="106" t="inlineStr"/>
+      <c r="E42" s="106" t="inlineStr"/>
+      <c r="F42" s="108" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G42" s="105" t="inlineStr">
+        <is>
+          <t>Adopt low-flow fixture standards for renovations/new build; document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="104" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="B43" s="105" t="inlineStr">
+        <is>
+          <t>Construction Activity Pollution Prevention</t>
+        </is>
+      </c>
+      <c r="C43" s="106" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="D43" s="106" t="inlineStr"/>
+      <c r="E43" s="106" t="inlineStr"/>
+      <c r="F43" s="108" t="inlineStr">
+        <is>
+          <t>N/A now</t>
+        </is>
+      </c>
+      <c r="G43" s="105" t="inlineStr">
+        <is>
+          <t>Applies to active construction. Require SWPPP/erosion control on future projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B44" s="105" t="inlineStr">
+        <is>
+          <t>Certified Green Buildings</t>
+        </is>
+      </c>
+      <c r="C44" s="106" t="n">
+        <v>5</v>
+      </c>
+      <c r="D44" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G44" s="105" t="inlineStr">
+        <is>
+          <t>Incentivize/require green certification for redevelopment (target the shopping-center &amp; corridor projects).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B45" s="105" t="inlineStr">
+        <is>
+          <t>Optimize Building Energy Performance</t>
+        </is>
+      </c>
+      <c r="C45" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G45" s="105" t="inlineStr">
+        <is>
+          <t>Efficiency retrofits; solar-ready + high-performance envelope standards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B46" s="105" t="inlineStr">
+        <is>
+          <t>Indoor Water Use Reduction</t>
+        </is>
+      </c>
+      <c r="C46" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G46" s="105" t="inlineStr">
+        <is>
+          <t>Low-flow fixture retrofit program.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B47" s="105" t="inlineStr">
+        <is>
+          <t>Outdoor Water Use Reduction</t>
+        </is>
+      </c>
+      <c r="C47" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="109" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="G47" s="105" t="inlineStr">
+        <is>
+          <t>Florida-Friendly landscaping, smart irrigation, native/xeric plantings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B48" s="105" t="inlineStr">
+        <is>
+          <t>Building Reuse</t>
+        </is>
+      </c>
+      <c r="C48" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="107" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="G48" s="105" t="inlineStr">
+        <is>
+          <t>Continue adaptive reuse over teardown where practical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B49" s="105" t="inlineStr">
+        <is>
+          <t>Historic Resource Preservation / Adaptive Reuse</t>
+        </is>
+      </c>
+      <c r="C49" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G49" s="105" t="inlineStr">
+        <is>
+          <t>Leverage Butler House / any historic structures; consider local historic designation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B50" s="105" t="inlineStr">
+        <is>
+          <t>Minimized Site Disturbance</t>
+        </is>
+      </c>
+      <c r="C50" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="108" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G50" s="105" t="inlineStr">
+        <is>
+          <t>Built-out. Applies to infill - protect soils &amp; trees on new construction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B51" s="105" t="inlineStr">
+        <is>
+          <t>Rainwater Management</t>
+        </is>
+      </c>
+      <c r="C51" s="106" t="n">
+        <v>4</v>
+      </c>
+      <c r="D51" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G51" s="105" t="inlineStr">
+        <is>
+          <t>Green stormwater infrastructure (bioswales, permeable paving) at the retail lot &amp; ROW; cut canal nutrient loading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B52" s="105" t="inlineStr">
+        <is>
+          <t>Heat Island Reduction</t>
+        </is>
+      </c>
+      <c r="C52" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="109" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="G52" s="105" t="inlineStr">
+        <is>
+          <t>Cool/permeable pavement, shade trees, reflective roofs at the shopping center.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B53" s="105" t="inlineStr">
+        <is>
+          <t>Solar Orientation</t>
+        </is>
+      </c>
+      <c r="C53" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="108" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G53" s="105" t="inlineStr">
+        <is>
+          <t>Applies to new layout; adopt solar-ready orientation for infill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B54" s="105" t="inlineStr">
+        <is>
+          <t>Renewable Energy Production</t>
+        </is>
+      </c>
+      <c r="C54" s="106" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G54" s="105" t="inlineStr">
+        <is>
+          <t>Rooftop / community-solar program; solar on the shopping-center roof.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B55" s="105" t="inlineStr">
+        <is>
+          <t>District Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="C55" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G55" s="105" t="inlineStr">
+        <is>
+          <t>Not viable at this scale - skip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B56" s="105" t="inlineStr">
+        <is>
+          <t>Infrastructure Energy Efficiency</t>
+        </is>
+      </c>
+      <c r="C56" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G56" s="105" t="inlineStr">
+        <is>
+          <t>LED streetlights; efficient pumps on canal/stormwater infrastructure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B57" s="105" t="inlineStr">
+        <is>
+          <t>Wastewater Management</t>
+        </is>
+      </c>
+      <c r="C57" s="106" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="109" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="G57" s="105" t="inlineStr">
+        <is>
+          <t>Explore greywater/reuse; nutrient reduction to protect the Intracoastal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B58" s="105" t="inlineStr">
+        <is>
+          <t>Recycled and Reused Infrastructure</t>
+        </is>
+      </c>
+      <c r="C58" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G58" s="105" t="inlineStr">
+        <is>
+          <t>Reuse road base/materials in future right-of-way projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B59" s="105" t="inlineStr">
+        <is>
+          <t>Solid Waste Management</t>
+        </is>
+      </c>
+      <c r="C59" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" s="107" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="G59" s="105" t="inlineStr">
+        <is>
+          <t>Maintain curbside recycling; add construction-waste diversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B60" s="105" t="inlineStr">
+        <is>
+          <t>Light Pollution Reduction</t>
+        </is>
+      </c>
+      <c r="C60" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G60" s="105" t="inlineStr">
+        <is>
+          <t>Dark-sky-compliant fixtures (important near the ICW / wildlife).</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="111" t="n"/>
+      <c r="B61" s="112" t="inlineStr">
+        <is>
+          <t>Subtotal - Green Infrastructure &amp; Buildings</t>
+        </is>
+      </c>
+      <c r="C61" s="102" t="n">
+        <v>31</v>
+      </c>
+      <c r="D61" s="102" t="n">
+        <v>2</v>
+      </c>
+      <c r="E61" s="102" t="n">
+        <v>5</v>
+      </c>
+      <c r="F61" s="111" t="n"/>
+      <c r="G61" s="111" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="103" t="inlineStr">
+        <is>
+          <t>INNOVATION &amp; DESIGN PROCESS (max 6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B63" s="105" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="C63" s="106" t="n">
+        <v>5</v>
+      </c>
+      <c r="D63" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G63" s="105" t="inlineStr">
+        <is>
+          <t>Pilot exemplary strategies (resilience / living shoreline / stormwater) for innovation points.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="A64" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B64" s="105" t="inlineStr">
+        <is>
+          <t>LEED Accredited Professional</t>
+        </is>
+      </c>
+      <c r="C64" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" s="110" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="G64" s="105" t="inlineStr">
+        <is>
+          <t>Put a LEED AP on any redevelopment team.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="111" t="n"/>
+      <c r="B65" s="112" t="inlineStr">
+        <is>
+          <t>Subtotal - Innovation &amp; Design Process</t>
+        </is>
+      </c>
+      <c r="C65" s="102" t="n">
+        <v>6</v>
+      </c>
+      <c r="D65" s="102" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" s="102" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" s="111" t="n"/>
+      <c r="G65" s="111" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="103" t="inlineStr">
+        <is>
+          <t>REGIONAL PRIORITY (max 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="30" customHeight="1">
+      <c r="A67" s="104" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="B67" s="105" t="inlineStr">
+        <is>
+          <t>Regional Priority (x4, Region Defined)</t>
+        </is>
+      </c>
+      <c r="C67" s="106" t="n">
+        <v>4</v>
+      </c>
+      <c r="D67" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" s="109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="G67" s="105" t="inlineStr">
+        <is>
+          <t>Pursue Florida-relevant RP credits (rainwater / heat island / water) once the underlying credits are achieved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="111" t="n"/>
+      <c r="B68" s="112" t="inlineStr">
+        <is>
+          <t>Subtotal - Regional Priority</t>
+        </is>
+      </c>
+      <c r="C68" s="102" t="n">
+        <v>4</v>
+      </c>
+      <c r="D68" s="102" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" s="102" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" s="111" t="n"/>
+      <c r="G68" s="111" t="n"/>
+    </row>
+    <row r="69" ht="24" customHeight="1">
+      <c r="A69" s="113" t="n"/>
+      <c r="B69" s="114" t="inlineStr">
+        <is>
+          <t>PROJECT TOTAL (interpretive)</t>
+        </is>
+      </c>
+      <c r="C69" s="115" t="n">
+        <v>110</v>
+      </c>
+      <c r="D69" s="116" t="n">
+        <v>20</v>
+      </c>
+      <c r="E69" s="116" t="n">
+        <v>38</v>
+      </c>
+      <c r="F69" s="117" t="inlineStr">
+        <is>
+          <t>&lt; Certified</t>
+        </is>
+      </c>
+      <c r="G69" s="118" t="inlineStr">
+        <is>
+          <t>Certified 40-49 | Silver 50-59 | Gold 60-79 | Platinum 80+</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="119" t="inlineStr">
+        <is>
+          <t>HOW IT SCORES NOW: ~20 points as-is  -&gt;  BELOW the 40-pt Certified floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="119" t="inlineStr">
+        <is>
+          <t>CEILING FROM THE ACTIONS LISTED ABOVE (conservative): ~38 points - still just short of Certified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="119" t="inlineStr">
+        <is>
+          <t>PATH TO CERTIFIED (40-49) / SILVER: the big swings are STRUCTURAL - rezone the US-1 &amp; Hillsboro EDGES for</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   mixed-use/higher density (Compact Development, Housing Types, Mixed-Use) and REQUIRE green building on new</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   construction (unlocks the GIB prerequisites + Certified Green Buildings + Energy). Those moves add ~15-25 pts over time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="119" t="inlineStr">
+        <is>
+          <t>REMINDER: LEED-ND certifies NEW development projects; this is an interpretive read of an existing neighborhood for planning use.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A74:G74"/>
+    <mergeCell ref="A70:G70"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A62:G62"/>
+    <mergeCell ref="A72:G72"/>
+    <mergeCell ref="A71:G71"/>
+    <mergeCell ref="A73:G73"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A75:G75"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AE106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
@@ -3265,7 +5382,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add 'Integrate Now - Qualify For' tab to Cove LEED-ND scorecard
Reframe from certification to as-is improvement: which LEED-ND credits The Cove
can realistically integrate/qualify for with no rezoning or new buildings,
tiered by effort and tied to programs Deerfield Beach/Broward already run
(Shady Street Tree program, NatureScape/Florida-Friendly, sea-turtle lighting
ordinance, FEMA CRS). ~30 points achievable as-is (Tier 1 ~10 in hand);
Tier 4 (redevelopment) flagged as informational only.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C83XSMHt5roS8jvvJWFf8j
</commit_message>
<xml_diff>
--- a/the_cove_deerfield_beach/the_cove_LEED_ND_scorecard.xlsx
+++ b/the_cove_deerfield_beach/the_cove_LEED_ND_scorecard.xlsx
@@ -6,13 +6,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="90" yWindow="450" windowWidth="12390" windowHeight="5085" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="The Cove - Scored + Actions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Neighborhood Development Plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Neighborhood Development" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Integrate Now - Qualify For" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="The Cove - Scored + Actions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Neighborhood Development Plan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Neighborhood Development" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Neighborhood Development Plan'!$A$1:$Q$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Neighborhood Development'!$A$1:$Q$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Neighborhood Development Plan'!$A$1:$Q$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Neighborhood Development'!$A$1:$Q$42</definedName>
   </definedNames>
   <calcPr calcId="145621" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="33">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -211,8 +212,12 @@
       <i val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -288,6 +293,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -434,7 +454,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -818,6 +838,49 @@
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="10" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="15" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="17" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1119,6 +1182,636 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="100" t="inlineStr">
+        <is>
+          <t>The Cove - Integrating LEED-ND As-Is: What We Can Qualify For (no certification required)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="101" t="inlineStr">
+        <is>
+          <t>LEED-ND Credit</t>
+        </is>
+      </c>
+      <c r="B2" s="102" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="C2" s="101" t="inlineStr">
+        <is>
+          <t>How to integrate into The Cove (as-is)</t>
+        </is>
+      </c>
+      <c r="D2" s="101" t="inlineStr">
+        <is>
+          <t>Why it improves the neighborhood</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="119" t="inlineStr">
+        <is>
+          <t>The question: not 'how do we get certified' but 'which LEED-ND ideas can we graft onto The Cove as-is to improve it - and what do we qualify for?'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="120" t="inlineStr">
+        <is>
+          <t>TIER 1  -  ALREADY QUALIFY / JUST DOCUMENT IT  (essentially in hand today)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="121" t="inlineStr">
+        <is>
+          <t>Access to Civic &amp; Public Space</t>
+        </is>
+      </c>
+      <c r="B6" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="123" t="inlineStr">
+        <is>
+          <t>Document Sullivan Park promenade + public waterfront access.</t>
+        </is>
+      </c>
+      <c r="D6" s="123" t="inlineStr">
+        <is>
+          <t>Protects &amp; showcases public waterfront - the neighborhood's signature asset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="121" t="inlineStr">
+        <is>
+          <t>Access to Recreation Facilities</t>
+        </is>
+      </c>
+      <c r="B7" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="123" t="inlineStr">
+        <is>
+          <t>Document walk/bike access to Sullivan Park, the pier, the beach, Deerfield Island shuttle.</t>
+        </is>
+      </c>
+      <c r="D7" s="123" t="inlineStr">
+        <is>
+          <t>Confirms The Cove as a recreation-rich district.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="121" t="inlineStr">
+        <is>
+          <t>Local Food Production</t>
+        </is>
+      </c>
+      <c r="B8" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="123" t="inlineStr">
+        <is>
+          <t>Recognize the Cove / Butler House farmers market; add a community-garden plot.</t>
+        </is>
+      </c>
+      <c r="D8" s="123" t="inlineStr">
+        <is>
+          <t>Local food + a recurring community gathering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="121" t="inlineStr">
+        <is>
+          <t>Neighborhood Schools</t>
+        </is>
+      </c>
+      <c r="B9" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="123" t="inlineStr">
+        <is>
+          <t>Document walkable access to St. Ambrose + Deerfield schools.</t>
+        </is>
+      </c>
+      <c r="D9" s="123" t="inlineStr">
+        <is>
+          <t>Supports walk-to-school &amp; family retention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="121" t="inlineStr">
+        <is>
+          <t>Transit Facilities</t>
+        </is>
+      </c>
+      <c r="B10" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="123" t="inlineStr">
+        <is>
+          <t>Inventory BCT stops/shelters on US-1 &amp; Hillsboro; add benches/real-time signs.</t>
+        </is>
+      </c>
+      <c r="D10" s="123" t="inlineStr">
+        <is>
+          <t>Makes the bus a real option at the edges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="121" t="inlineStr">
+        <is>
+          <t>Building Reuse</t>
+        </is>
+      </c>
+      <c r="B11" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="123" t="inlineStr">
+        <is>
+          <t>Adopt a 'reuse-over-teardown' preference for existing homes.</t>
+        </is>
+      </c>
+      <c r="D11" s="123" t="inlineStr">
+        <is>
+          <t>Keeps neighborhood character &amp; embodied carbon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="121" t="inlineStr">
+        <is>
+          <t>Solid Waste Management</t>
+        </is>
+      </c>
+      <c r="B12" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="123" t="inlineStr">
+        <is>
+          <t>Document the city curbside recycling program; add construction-waste diversion.</t>
+        </is>
+      </c>
+      <c r="D12" s="123" t="inlineStr">
+        <is>
+          <t>Cleaner waste stream, little cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="121" t="inlineStr">
+        <is>
+          <t>Light Pollution Reduction</t>
+        </is>
+      </c>
+      <c r="B13" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="123" t="inlineStr">
+        <is>
+          <t>Deerfield ALREADY enforces a sea-turtle/coastal lighting ordinance (Broward Beach Lighting Mgmt Plan) - extend fixture standards inland.</t>
+        </is>
+      </c>
+      <c r="D13" s="123" t="inlineStr">
+        <is>
+          <t>Dark-sky, wildlife-friendly, safer streets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="121" t="inlineStr">
+        <is>
+          <t>Community Outreach &amp; Involvement</t>
+        </is>
+      </c>
+      <c r="B14" s="122" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="123" t="inlineStr">
+        <is>
+          <t>Formalize a charrette/engagement process with the active Cove Civic Association.</t>
+        </is>
+      </c>
+      <c r="D14" s="123" t="inlineStr">
+        <is>
+          <t>Gives residents a real seat at planning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="112" t="inlineStr">
+        <is>
+          <t>Subtotal - Tier 1 (in hand / document)</t>
+        </is>
+      </c>
+      <c r="B15" s="102" t="n">
+        <v>10</v>
+      </c>
+      <c r="C15" s="111" t="n"/>
+      <c r="D15" s="111" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="124" t="inlineStr">
+        <is>
+          <t>TIER 2  -  PLUG INTO A PROGRAM THE CITY/COUNTY ALREADY RUNS  (low cost, high benefit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="125" t="inlineStr">
+        <is>
+          <t>Tree-Lined &amp; Shaded Streetscapes</t>
+        </is>
+      </c>
+      <c r="B18" s="126" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="127" t="inlineStr">
+        <is>
+          <t>Deploy Deerfield's 'Shady Street Tree' cost-share + free tree giveaways + $50-100 rebates, street by street.</t>
+        </is>
+      </c>
+      <c r="D18" s="127" t="inlineStr">
+        <is>
+          <t>Shade, cooler walks, curb appeal, stormwater help.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="125" t="inlineStr">
+        <is>
+          <t>Outdoor Water Use Reduction</t>
+        </is>
+      </c>
+      <c r="B19" s="126" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="127" t="inlineStr">
+        <is>
+          <t>Enroll The Cove in Broward NatureScape / Florida-Friendly Landscaping (Silver/Gold); native + smart irrigation.</t>
+        </is>
+      </c>
+      <c r="D19" s="127" t="inlineStr">
+        <is>
+          <t>Lower water bills; less fertilizer/runoff into the canals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="125" t="inlineStr">
+        <is>
+          <t>Heat Island Reduction</t>
+        </is>
+      </c>
+      <c r="B20" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="127" t="inlineStr">
+        <is>
+          <t>Pair the tree canopy with light/permeable surfaces at the shopping-center lot &amp; rights-of-way.</t>
+        </is>
+      </c>
+      <c r="D20" s="127" t="inlineStr">
+        <is>
+          <t>Cooler, more comfortable public realm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="125" t="inlineStr">
+        <is>
+          <t>Bicycle Facilities</t>
+        </is>
+      </c>
+      <c r="B21" s="126" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="127" t="inlineStr">
+        <is>
+          <t>Add bike racks at the Cove node + connect to the county bike/greenway network toward the beach.</t>
+        </is>
+      </c>
+      <c r="D21" s="127" t="inlineStr">
+        <is>
+          <t>Safer biking to shops, park, beach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="112" t="inlineStr">
+        <is>
+          <t>Subtotal - Tier 2 (existing programs)</t>
+        </is>
+      </c>
+      <c r="B22" s="102" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" s="111" t="n"/>
+      <c r="D22" s="111" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="128" t="inlineStr">
+        <is>
+          <t>TIER 3  -  A CAPITAL / STREETSCAPE PROJECT OR ANALYSIS  (budget yes, rezoning NO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="129" t="inlineStr">
+        <is>
+          <t>Preferred Locations</t>
+        </is>
+      </c>
+      <c r="B25" s="130" t="n">
+        <v>7</v>
+      </c>
+      <c r="C25" s="131" t="inlineStr">
+        <is>
+          <t>Already a qualifying infill location - commission the connectivity/adjacency analysis to claim it.</t>
+        </is>
+      </c>
+      <c r="D25" s="131" t="inlineStr">
+        <is>
+          <t>Formalizes The Cove's 'smart location' story for grants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="129" t="inlineStr">
+        <is>
+          <t>Walkable Streets</t>
+        </is>
+      </c>
+      <c r="B26" s="130" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" s="131" t="inlineStr">
+        <is>
+          <t>Sidewalk gap-fill, marked crossings, traffic calming, street trees on the grid + corridors.</t>
+        </is>
+      </c>
+      <c r="D26" s="131" t="inlineStr">
+        <is>
+          <t>Safer, more walkable everyday streets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="129" t="inlineStr">
+        <is>
+          <t>Access to Quality Transit</t>
+        </is>
+      </c>
+      <c r="B27" s="130" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" s="131" t="inlineStr">
+        <is>
+          <t>Advocate higher BCT frequency on US-1/Hillsboro; upgrade shelters; document service.</t>
+        </is>
+      </c>
+      <c r="D27" s="131" t="inlineStr">
+        <is>
+          <t>Better mobility without a car.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="42" customHeight="1">
+      <c r="A28" s="129" t="inlineStr">
+        <is>
+          <t>Housing &amp; Jobs Proximity</t>
+        </is>
+      </c>
+      <c r="B28" s="130" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" s="131" t="inlineStr">
+        <is>
+          <t>Document jobs within 1/2 mile (Cove retail + Hillsboro corridor).</t>
+        </is>
+      </c>
+      <c r="D28" s="131" t="inlineStr">
+        <is>
+          <t>Confirms a real live-work balance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="42" customHeight="1">
+      <c r="A29" s="129" t="inlineStr">
+        <is>
+          <t>Rainwater Management</t>
+        </is>
+      </c>
+      <c r="B29" s="130" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="131" t="inlineStr">
+        <is>
+          <t>Green stormwater (bioswales, permeable paving) at the retail lot &amp; ROW; build on the city's FEMA-CRS floodplain program.</t>
+        </is>
+      </c>
+      <c r="D29" s="131" t="inlineStr">
+        <is>
+          <t>Less flooding + cleaner canal/ICW water.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="129" t="inlineStr">
+        <is>
+          <t>Historic Resource Preservation</t>
+        </is>
+      </c>
+      <c r="B30" s="130" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="131" t="inlineStr">
+        <is>
+          <t>Leverage the Butler House / consider a local historic designation.</t>
+        </is>
+      </c>
+      <c r="D30" s="131" t="inlineStr">
+        <is>
+          <t>Protects heritage; opens preservation grants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="112" t="inlineStr">
+        <is>
+          <t>Subtotal - Tier 3 (capital / analysis)</t>
+        </is>
+      </c>
+      <c r="B31" s="102" t="n">
+        <v>18</v>
+      </c>
+      <c r="C31" s="111" t="n"/>
+      <c r="D31" s="111" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="132" t="inlineStr">
+        <is>
+          <t>TIER 4  -  ONLY WITH REDEVELOPMENT / NEW BUILDINGS  (not now - this is where certification really lives)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="133" t="inlineStr">
+        <is>
+          <t>Compact Development / Housing Types / Mixed-Use</t>
+        </is>
+      </c>
+      <c r="B34" s="134" t="n">
+        <v>17</v>
+      </c>
+      <c r="C34" s="135" t="inlineStr">
+        <is>
+          <t>Would require rezoning the US-1 &amp; Hillsboro EDGES for mixed-use + higher density.</t>
+        </is>
+      </c>
+      <c r="D34" s="135" t="inlineStr">
+        <is>
+          <t>Biggest point block AND biggest change - a separate policy decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" s="133" t="inlineStr">
+        <is>
+          <t>Certified Green Buildings / Energy / Renewables</t>
+        </is>
+      </c>
+      <c r="B35" s="134" t="n">
+        <v>12</v>
+      </c>
+      <c r="C35" s="135" t="inlineStr">
+        <is>
+          <t>Would require a green-building requirement + retrofits on new construction.</t>
+        </is>
+      </c>
+      <c r="D35" s="135" t="inlineStr">
+        <is>
+          <t>Unlocks the GIB prerequisites over time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" s="133" t="inlineStr">
+        <is>
+          <t>Reduced Parking / TDM</t>
+        </is>
+      </c>
+      <c r="B36" s="134" t="inlineStr">
+        <is>
+          <t>3+</t>
+        </is>
+      </c>
+      <c r="C36" s="135" t="inlineStr">
+        <is>
+          <t>Tied to redevelopment of the shopping-center site.</t>
+        </is>
+      </c>
+      <c r="D36" s="135" t="inlineStr">
+        <is>
+          <t>Only makes sense with a redevelopment project.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="112" t="inlineStr">
+        <is>
+          <t>Subtotal - Tier 4 (needs redevelopment - informational)</t>
+        </is>
+      </c>
+      <c r="B37" s="102" t="n">
+        <v>29</v>
+      </c>
+      <c r="C37" s="111" t="n"/>
+      <c r="D37" s="111" t="n"/>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="136" t="inlineStr">
+        <is>
+          <t>ACHIEVABLE WITH NO REZONING / NO NEW BUILDINGS (Tiers 1-3):  ~30 points  |  Tier 1 (~10) is essentially in hand now</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="119" t="inlineStr">
+        <is>
+          <t>BOTTOM LINE: with NO rezoning and NO new buildings, The Cove can realistically integrate/qualify for ~30 points of LEED-ND strategies -</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Tier 1 (~10) is essentially in hand today; Tiers 2-3 add ~20 more through existing city/county programs and streetscape projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Every one of these is a genuine neighborhood improvement (shade, water, stormwater, walk/bike, wildlife lighting, public waterfront) - the points are a bonus, not the goal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   The jump PAST ~30 toward Certified (40) is Tier 4 - a deliberate redevelopment/rezoning choice for the US-1 &amp; Hillsboro edges, not an as-is improvement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="119" t="inlineStr">
+        <is>
+          <t>Local programs referenced: Deerfield Beach Tree Programs (Shady Street Tree, giveaways, rebates); Broward NatureScape / Florida-Friendly Landscaping; Deerfield sea-turtle lighting ordinance; FEMA Community Rating System (city participant).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A44:D44"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3105,7 +3798,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5382,7 +6075,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add Year 1-3 action plan tab to Cove LEED-ND scorecard
Phased integration plan (Document & quick wins -> programs -> capital projects)
with the LEED-ND credit(s) earned, lead/owner, and rough cost per action, tied
to real Deerfield/Broward programs. Cumulative ~33 pts with no rezoning
(Yr1 ~10, Yr2 ~24, Yr3 ~33); Tier-4 policy track (edge rezoning + green-building
requirement) flagged as the separate path toward Certified.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C83XSMHt5roS8jvvJWFf8j
</commit_message>
<xml_diff>
--- a/the_cove_deerfield_beach/the_cove_LEED_ND_scorecard.xlsx
+++ b/the_cove_deerfield_beach/the_cove_LEED_ND_scorecard.xlsx
@@ -6,14 +6,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="90" yWindow="450" windowWidth="12390" windowHeight="5085" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Integrate Now - Qualify For" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="The Cove - Scored + Actions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Neighborhood Development Plan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Neighborhood Development" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Action Plan (Yr 1-3)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Integrate Now - Qualify For" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="The Cove - Scored + Actions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Neighborhood Development Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Neighborhood Development" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Neighborhood Development Plan'!$A$1:$Q$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Neighborhood Development'!$A$1:$Q$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Neighborhood Development Plan'!$A$1:$Q$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Neighborhood Development'!$A$1:$Q$42</definedName>
   </definedNames>
   <calcPr calcId="145621" fullCalcOnLoad="1"/>
 </workbook>
@@ -311,7 +312,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -450,11 +451,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="140">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -882,6 +927,9 @@
     <xf numFmtId="0" fontId="31" fillId="14" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="9" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1182,6 +1230,748 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="100" t="inlineStr">
+        <is>
+          <t>The Cove - LEED-ND Integration Action Plan (Year 1-3) with Credits Earned</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="101" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="B2" s="101" t="inlineStr">
+        <is>
+          <t>LEED-ND credit(s) earned</t>
+        </is>
+      </c>
+      <c r="C2" s="102" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="D2" s="101" t="inlineStr">
+        <is>
+          <t>Lead / Owner</t>
+        </is>
+      </c>
+      <c r="E2" s="102" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="F2" s="101" t="inlineStr">
+        <is>
+          <t>Neighborhood benefit</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="119" t="inlineStr">
+        <is>
+          <t>Phased plan to graft LEED-ND value into The Cove as-is. Cost key: $ = staff time/&lt;$5k | $$ = cost-share/study/$5-50k | $$$ = capital $50k+ | policy = process, not $$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="120" t="inlineStr">
+        <is>
+          <t>YEAR 1  -  DOCUMENT &amp; QUICK WINS  (mostly free; claim what's already true)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="121" t="inlineStr">
+        <is>
+          <t>Compile a neighborhood 'asset dossier' (parks, pier, farmers market, schools, bus stops, recycling)</t>
+        </is>
+      </c>
+      <c r="B6" s="123" t="inlineStr">
+        <is>
+          <t>Civic Space; Recreation; Local Food; Schools; Transit Facilities; Solid Waste</t>
+        </is>
+      </c>
+      <c r="C6" s="122" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" s="123" t="inlineStr">
+        <is>
+          <t>City Planning + Cove Civic Assoc.</t>
+        </is>
+      </c>
+      <c r="E6" s="122" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F6" s="123" t="inlineStr">
+        <is>
+          <t>Claims 6 credits already true; produces a grant-ready asset map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="121" t="inlineStr">
+        <is>
+          <t>Adopt a 'reuse-over-teardown' preference for existing homes</t>
+        </is>
+      </c>
+      <c r="B7" s="123" t="inlineStr">
+        <is>
+          <t>Building Reuse</t>
+        </is>
+      </c>
+      <c r="C7" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="123" t="inlineStr">
+        <is>
+          <t>Planning / Building Dept.</t>
+        </is>
+      </c>
+      <c r="E7" s="122" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F7" s="123" t="inlineStr">
+        <is>
+          <t>Preserves neighborhood character &amp; embodied carbon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="121" t="inlineStr">
+        <is>
+          <t>Formalize a resident engagement process (regular charrettes) with the Cove Civic Assoc.</t>
+        </is>
+      </c>
+      <c r="B8" s="123" t="inlineStr">
+        <is>
+          <t>Community Outreach &amp; Involvement</t>
+        </is>
+      </c>
+      <c r="C8" s="122" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="123" t="inlineStr">
+        <is>
+          <t>Cove Civic Assoc. + Planning</t>
+        </is>
+      </c>
+      <c r="E8" s="122" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F8" s="123" t="inlineStr">
+        <is>
+          <t>Residents get a standing seat at planning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="121" t="inlineStr">
+        <is>
+          <t>Extend the sea-turtle / dark-sky lighting standard inland; begin fixture swaps</t>
+        </is>
+      </c>
+      <c r="B9" s="123" t="inlineStr">
+        <is>
+          <t>Light Pollution Reduction</t>
+        </is>
+      </c>
+      <c r="C9" s="122" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="123" t="inlineStr">
+        <is>
+          <t>Public Works / Code Enforcement</t>
+        </is>
+      </c>
+      <c r="E9" s="122" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="F9" s="123" t="inlineStr">
+        <is>
+          <t>Safer, wildlife-friendly nights (city ordinance already exists).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="121" t="inlineStr">
+        <is>
+          <t>Kick off street-tree planting via Deerfield's Shady Street Tree program + Arbor Day giveaways</t>
+        </is>
+      </c>
+      <c r="B10" s="123" t="inlineStr">
+        <is>
+          <t>(starts Tree-Lined &amp; Heat Island - credited Yr 2)</t>
+        </is>
+      </c>
+      <c r="C10" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="123" t="inlineStr">
+        <is>
+          <t>Environmental Services + residents</t>
+        </is>
+      </c>
+      <c r="E10" s="122" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="F10" s="123" t="inlineStr">
+        <is>
+          <t>Shade &amp; cooling underway at cost-share pricing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="121" t="inlineStr">
+        <is>
+          <t>Enroll the neighborhood in Broward NatureScape / Florida-Friendly Landscaping</t>
+        </is>
+      </c>
+      <c r="B11" s="123" t="inlineStr">
+        <is>
+          <t>(starts Outdoor Water - credited Yr 2)</t>
+        </is>
+      </c>
+      <c r="C11" s="122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="123" t="inlineStr">
+        <is>
+          <t>Cove Civic Assoc. + UF/IFAS Broward</t>
+        </is>
+      </c>
+      <c r="E11" s="122" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F11" s="123" t="inlineStr">
+        <is>
+          <t>Water savings &amp; cleaner canal runoff begin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="112" t="inlineStr">
+        <is>
+          <t>Year 1 subtotal</t>
+        </is>
+      </c>
+      <c r="B12" s="137" t="inlineStr">
+        <is>
+          <t>credits earned this year</t>
+        </is>
+      </c>
+      <c r="C12" s="102" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="111" t="n"/>
+      <c r="E12" s="111" t="n"/>
+      <c r="F12" s="111" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="124" t="inlineStr">
+        <is>
+          <t>YEAR 2  -  PROGRAMS MATURE + FIRST ANALYSES  (low-moderate cost)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="125" t="inlineStr">
+        <is>
+          <t>Reach street-tree canopy / shading targets (continue the program)</t>
+        </is>
+      </c>
+      <c r="B15" s="127" t="inlineStr">
+        <is>
+          <t>Tree-Lined &amp; Shaded Streetscapes; Heat Island Reduction</t>
+        </is>
+      </c>
+      <c r="C15" s="126" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="127" t="inlineStr">
+        <is>
+          <t>Environmental Services</t>
+        </is>
+      </c>
+      <c r="E15" s="126" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="F15" s="127" t="inlineStr">
+        <is>
+          <t>Cooler, shadier, more walkable streets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="44" customHeight="1">
+      <c r="A16" s="125" t="inlineStr">
+        <is>
+          <t>Achieve NatureScape Silver/Gold recognition (native + smart irrigation)</t>
+        </is>
+      </c>
+      <c r="B16" s="127" t="inlineStr">
+        <is>
+          <t>Outdoor Water Use Reduction</t>
+        </is>
+      </c>
+      <c r="C16" s="126" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="127" t="inlineStr">
+        <is>
+          <t>Cove Civic Assoc. + UF/IFAS</t>
+        </is>
+      </c>
+      <c r="E16" s="126" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F16" s="127" t="inlineStr">
+        <is>
+          <t>Lower water bills; less fertilizer into the ICW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="44" customHeight="1">
+      <c r="A17" s="125" t="inlineStr">
+        <is>
+          <t>Install bike racks + first bike-lane/greenway links (Cove node -&gt; beach &amp; park)</t>
+        </is>
+      </c>
+      <c r="B17" s="127" t="inlineStr">
+        <is>
+          <t>Bicycle Facilities</t>
+        </is>
+      </c>
+      <c r="C17" s="126" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="127" t="inlineStr">
+        <is>
+          <t>City + Broward MPO</t>
+        </is>
+      </c>
+      <c r="E17" s="126" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="F17" s="127" t="inlineStr">
+        <is>
+          <t>Safe biking to shops, park, beach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="44" customHeight="1">
+      <c r="A18" s="125" t="inlineStr">
+        <is>
+          <t>Commission a connectivity/adjacency + jobs-proximity study</t>
+        </is>
+      </c>
+      <c r="B18" s="127" t="inlineStr">
+        <is>
+          <t>Preferred Locations; Housing &amp; Jobs Proximity</t>
+        </is>
+      </c>
+      <c r="C18" s="126" t="n">
+        <v>7</v>
+      </c>
+      <c r="D18" s="127" t="inlineStr">
+        <is>
+          <t>Planning + consultant</t>
+        </is>
+      </c>
+      <c r="E18" s="126" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="F18" s="127" t="inlineStr">
+        <is>
+          <t>Formalizes the 'smart location' story; grant-ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="125" t="inlineStr">
+        <is>
+          <t>Begin BCT service advocacy + shelter design</t>
+        </is>
+      </c>
+      <c r="B19" s="127" t="inlineStr">
+        <is>
+          <t>(starts Access to Transit - credited Yr 3)</t>
+        </is>
+      </c>
+      <c r="C19" s="126" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="127" t="inlineStr">
+        <is>
+          <t>City + Broward County Transit</t>
+        </is>
+      </c>
+      <c r="E19" s="126" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="F19" s="127" t="inlineStr">
+        <is>
+          <t>Builds the pipeline to better bus service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
+      <c r="A20" s="125" t="inlineStr">
+        <is>
+          <t>Sidewalk-gap audit + priority crossing design</t>
+        </is>
+      </c>
+      <c r="B20" s="127" t="inlineStr">
+        <is>
+          <t>(starts Walkable Streets - credited Yr 3)</t>
+        </is>
+      </c>
+      <c r="C20" s="126" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="127" t="inlineStr">
+        <is>
+          <t>Engineering / Public Works</t>
+        </is>
+      </c>
+      <c r="E20" s="126" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="F20" s="127" t="inlineStr">
+        <is>
+          <t>A prioritized walk-safety plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="112" t="inlineStr">
+        <is>
+          <t>Year 2 subtotal</t>
+        </is>
+      </c>
+      <c r="B21" s="137" t="inlineStr">
+        <is>
+          <t>credits earned this year</t>
+        </is>
+      </c>
+      <c r="C21" s="102" t="n">
+        <v>14</v>
+      </c>
+      <c r="D21" s="111" t="n"/>
+      <c r="E21" s="111" t="n"/>
+      <c r="F21" s="111" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="128" t="inlineStr">
+        <is>
+          <t>YEAR 3  -  CAPITAL PROJECTS &amp; GREEN INFRASTRUCTURE  (budget required; still NO rezoning)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="44" customHeight="1">
+      <c r="A24" s="129" t="inlineStr">
+        <is>
+          <t>Build sidewalk / crossing / traffic-calming improvements</t>
+        </is>
+      </c>
+      <c r="B24" s="131" t="inlineStr">
+        <is>
+          <t>Walkable Streets</t>
+        </is>
+      </c>
+      <c r="C24" s="130" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" s="131" t="inlineStr">
+        <is>
+          <t>Public Works / Engineering</t>
+        </is>
+      </c>
+      <c r="E24" s="130" t="inlineStr">
+        <is>
+          <t>$$$</t>
+        </is>
+      </c>
+      <c r="F24" s="131" t="inlineStr">
+        <is>
+          <t>Safer everyday walking on the grid &amp; corridors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="44" customHeight="1">
+      <c r="A25" s="129" t="inlineStr">
+        <is>
+          <t>Green stormwater retrofit at the shopping-center lot &amp; ROW (bioswales, permeable paving)</t>
+        </is>
+      </c>
+      <c r="B25" s="131" t="inlineStr">
+        <is>
+          <t>Rainwater Management</t>
+        </is>
+      </c>
+      <c r="C25" s="130" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="131" t="inlineStr">
+        <is>
+          <t>Engineering / Stormwater</t>
+        </is>
+      </c>
+      <c r="E25" s="130" t="inlineStr">
+        <is>
+          <t>$$$</t>
+        </is>
+      </c>
+      <c r="F25" s="131" t="inlineStr">
+        <is>
+          <t>Less flooding, cleaner canal/ICW water; logs for FEMA CRS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="44" customHeight="1">
+      <c r="A26" s="129" t="inlineStr">
+        <is>
+          <t>Deliver higher BCT frequency + upgraded shelters</t>
+        </is>
+      </c>
+      <c r="B26" s="131" t="inlineStr">
+        <is>
+          <t>Access to Quality Transit</t>
+        </is>
+      </c>
+      <c r="C26" s="130" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="131" t="inlineStr">
+        <is>
+          <t>Broward County Transit + City</t>
+        </is>
+      </c>
+      <c r="E26" s="130" t="inlineStr">
+        <is>
+          <t>$$$</t>
+        </is>
+      </c>
+      <c r="F26" s="131" t="inlineStr">
+        <is>
+          <t>A real car-optional mobility option.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="44" customHeight="1">
+      <c r="A27" s="129" t="inlineStr">
+        <is>
+          <t>Pursue Butler House / a local historic designation</t>
+        </is>
+      </c>
+      <c r="B27" s="131" t="inlineStr">
+        <is>
+          <t>Historic Resource Preservation</t>
+        </is>
+      </c>
+      <c r="C27" s="130" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="131" t="inlineStr">
+        <is>
+          <t>Planning + Deerfield Historical Society</t>
+        </is>
+      </c>
+      <c r="E27" s="130" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="F27" s="131" t="inlineStr">
+        <is>
+          <t>Protects heritage; opens preservation grants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="112" t="inlineStr">
+        <is>
+          <t>Year 3 subtotal</t>
+        </is>
+      </c>
+      <c r="B28" s="137" t="inlineStr">
+        <is>
+          <t>credits earned this year</t>
+        </is>
+      </c>
+      <c r="C28" s="102" t="n">
+        <v>9</v>
+      </c>
+      <c r="D28" s="111" t="n"/>
+      <c r="E28" s="111" t="n"/>
+      <c r="F28" s="111" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="132" t="inlineStr">
+        <is>
+          <t>ONGOING / FUTURE  -  TIER 4 POLICY TRACK  (not counted below - this is the path PAST ~33 toward Certified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="44" customHeight="1">
+      <c r="A31" s="133" t="inlineStr">
+        <is>
+          <t>US-1 &amp; Hillsboro EDGE rezoning / mixed-use + higher-density study</t>
+        </is>
+      </c>
+      <c r="B31" s="135" t="inlineStr">
+        <is>
+          <t>Compact Development; Housing Types &amp; Affordability; Mixed-Use</t>
+        </is>
+      </c>
+      <c r="C31" s="134" t="inlineStr">
+        <is>
+          <t>~17</t>
+        </is>
+      </c>
+      <c r="D31" s="135" t="inlineStr">
+        <is>
+          <t>Planning + CRA + City Commission</t>
+        </is>
+      </c>
+      <c r="E31" s="134" t="inlineStr">
+        <is>
+          <t>policy/$$</t>
+        </is>
+      </c>
+      <c r="F31" s="135" t="inlineStr">
+        <is>
+          <t>Biggest point block AND biggest change - a deliberate policy decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="44" customHeight="1">
+      <c r="A32" s="133" t="inlineStr">
+        <is>
+          <t>Green-building requirement + retrofit incentives for new construction</t>
+        </is>
+      </c>
+      <c r="B32" s="135" t="inlineStr">
+        <is>
+          <t>Certified Green Buildings; Energy; Renewables</t>
+        </is>
+      </c>
+      <c r="C32" s="134" t="inlineStr">
+        <is>
+          <t>~12</t>
+        </is>
+      </c>
+      <c r="D32" s="135" t="inlineStr">
+        <is>
+          <t>City Commission / Building Dept.</t>
+        </is>
+      </c>
+      <c r="E32" s="134" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="F32" s="135" t="inlineStr">
+        <is>
+          <t>Unlocks the GIB prerequisites needed for actual certification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="136" t="inlineStr">
+        <is>
+          <t>TOTAL INTEGRATED WITH NO REZONING / NO NEW BUILDINGS:  ~33 LEED-ND points over 3 years</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="119" t="inlineStr">
+        <is>
+          <t>CUMULATIVE (no rezoning, no new buildings):  end of Yr 1 ~10 pts  -&gt;  end of Yr 2 ~24  -&gt;  end of Yr 3 ~33 pts of LEED-ND value integrated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="119" t="inlineStr">
+        <is>
+          <t>Every action is a real improvement (shade, water, stormwater, walk/bike, wildlife lighting, public waterfront) - the credits are the scorecard, not the goal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="119" t="inlineStr">
+        <is>
+          <t>To cross from ~33 into Certified (40-49) / Silver: pursue the Tier-4 policy track (edge rezoning + green-building requirement) as a separate Commission/CRA decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="119" t="inlineStr">
+        <is>
+          <t>Points are interpretive estimates; confirm specifics with Deerfield Beach Planning &amp; Zoning / GIS and Environmental Services before adopting.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A30:F30"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1233,6 +2023,9 @@
           <t>TIER 1  -  ALREADY QUALIFY / JUST DOCUMENT IT  (essentially in hand today)</t>
         </is>
       </c>
+      <c r="B5" s="138" t="n"/>
+      <c r="C5" s="138" t="n"/>
+      <c r="D5" s="139" t="n"/>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="121" t="inlineStr">
@@ -1432,6 +2225,9 @@
           <t>TIER 2  -  PLUG INTO A PROGRAM THE CITY/COUNTY ALREADY RUNS  (low cost, high benefit)</t>
         </is>
       </c>
+      <c r="B17" s="138" t="n"/>
+      <c r="C17" s="138" t="n"/>
+      <c r="D17" s="139" t="n"/>
     </row>
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="125" t="inlineStr">
@@ -1531,6 +2327,9 @@
           <t>TIER 3  -  A CAPITAL / STREETSCAPE PROJECT OR ANALYSIS  (budget yes, rezoning NO)</t>
         </is>
       </c>
+      <c r="B24" s="138" t="n"/>
+      <c r="C24" s="138" t="n"/>
+      <c r="D24" s="139" t="n"/>
     </row>
     <row r="25" ht="42" customHeight="1">
       <c r="A25" s="129" t="inlineStr">
@@ -1670,6 +2469,9 @@
           <t>TIER 4  -  ONLY WITH REDEVELOPMENT / NEW BUILDINGS  (not now - this is where certification really lives)</t>
         </is>
       </c>
+      <c r="B33" s="138" t="n"/>
+      <c r="C33" s="138" t="n"/>
+      <c r="D33" s="139" t="n"/>
     </row>
     <row r="34" ht="42" customHeight="1">
       <c r="A34" s="133" t="inlineStr">
@@ -1751,6 +2553,9 @@
           <t>ACHIEVABLE WITH NO REZONING / NO NEW BUILDINGS (Tiers 1-3):  ~30 points  |  Tier 1 (~10) is essentially in hand now</t>
         </is>
       </c>
+      <c r="B39" s="138" t="n"/>
+      <c r="C39" s="138" t="n"/>
+      <c r="D39" s="139" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="119" t="inlineStr">
@@ -1790,9 +2595,9 @@
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A5:D5"/>
     <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A40:D40"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A39:D39"/>
     <mergeCell ref="A43:D43"/>
@@ -1806,7 +2611,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3798,7 +4603,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6075,7 +6880,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Re-anchor to official Cove Waterfront District boundary + add master crosswalk
- Extract the provided 'Cove Waterfront District Study Area' from the supplied
  KMZ (32 vertices, ~1,040 acres / 1.63 sq mi) and generate authoritative
  boundary files (generate_study_area_files.py -> KML/GeoJSON/CSV). This
  supersedes the earlier interpretive polygon (~814 acres); it extends north of
  Hillsboro Blvd to the north waterfront.
- Add 'Master Crosswalk & Analysis' tab: all 56 official LEED-ND line items
  transposed against our analysis (Now/Achievable/Status/Tier/Timeline/Owner/
  Cost/Action) with an AutoFilter. Now ~20, achievable-without-rezoning ~39.
- Note the boundary supersession in source_notes.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C83XSMHt5roS8jvvJWFf8j
</commit_message>
<xml_diff>
--- a/the_cove_deerfield_beach/the_cove_LEED_ND_scorecard.xlsx
+++ b/the_cove_deerfield_beach/the_cove_LEED_ND_scorecard.xlsx
@@ -6,15 +6,17 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="90" yWindow="450" windowWidth="12390" windowHeight="5085" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Action Plan (Yr 1-3)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Integrate Now - Qualify For" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="The Cove - Scored + Actions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Neighborhood Development Plan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Neighborhood Development" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Master Crosswalk &amp; Analysis" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Action Plan (Yr 1-3)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Integrate Now - Qualify For" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="The Cove - Scored + Actions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Neighborhood Development Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Neighborhood Development" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Neighborhood Development Plan'!$A$1:$Q$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Neighborhood Development'!$A$1:$Q$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master Crosswalk &amp; Analysis'!$A$3:$L$59</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Neighborhood Development Plan'!$A$1:$Q$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Neighborhood Development'!$A$1:$Q$42</definedName>
   </definedNames>
   <calcPr calcId="145621" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="34">
+  <fonts count="38">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -217,8 +219,22 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -311,8 +327,13 @@
         <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -495,11 +516,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -930,6 +965,58 @@
     <xf numFmtId="0" fontId="32" fillId="9" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="10" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="10" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="12" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="16" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="18" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="18" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="15" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="17" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1230,6 +1317,3384 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L73"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="100" t="inlineStr">
+        <is>
+          <t>The Cove / Cove Waterfront District - LEED-ND Rating System crosswalked to our analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="140" t="inlineStr">
+        <is>
+          <t>Study area: Cove Waterfront District (official boundary from supplied KMZ, ~1,040 acres / 1.63 sq mi).  Each row = one official LEED-ND line item; use the AutoFilter to sort by Tier / Status / Category / Timeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="141" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B3" s="141" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C3" s="141" t="inlineStr">
+        <is>
+          <t>LEED-ND Item (official)</t>
+        </is>
+      </c>
+      <c r="D3" s="142" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="E3" s="142" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="F3" s="142" t="inlineStr">
+        <is>
+          <t>Poten- tial</t>
+        </is>
+      </c>
+      <c r="G3" s="141" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H3" s="141" t="inlineStr">
+        <is>
+          <t>Feasibility tier</t>
+        </is>
+      </c>
+      <c r="I3" s="141" t="inlineStr">
+        <is>
+          <t>Timeline</t>
+        </is>
+      </c>
+      <c r="J3" s="141" t="inlineStr">
+        <is>
+          <t>Lead / Owner</t>
+        </is>
+      </c>
+      <c r="K3" s="141" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="L3" s="141" t="inlineStr">
+        <is>
+          <t>Action / how to integrate</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B4" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C4" s="144" t="inlineStr">
+        <is>
+          <t>Smart Location</t>
+        </is>
+      </c>
+      <c r="D4" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E4" s="143" t="inlineStr"/>
+      <c r="F4" s="143" t="inlineStr"/>
+      <c r="G4" s="145" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="H4" s="146" t="inlineStr">
+        <is>
+          <t>1 In hand</t>
+        </is>
+      </c>
+      <c r="I4" s="147" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="J4" s="144" t="inlineStr">
+        <is>
+          <t>City Planning</t>
+        </is>
+      </c>
+      <c r="K4" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L4" s="144" t="inlineStr">
+        <is>
+          <t>Infill location qualifies; document adjacency/connectivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B5" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C5" s="144" t="inlineStr">
+        <is>
+          <t>Imperiled Species &amp; Ecological Communities</t>
+        </is>
+      </c>
+      <c r="D5" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E5" s="143" t="inlineStr"/>
+      <c r="F5" s="143" t="inlineStr"/>
+      <c r="G5" s="145" t="inlineStr">
+        <is>
+          <t>Met (verify)</t>
+        </is>
+      </c>
+      <c r="H5" s="146" t="inlineStr">
+        <is>
+          <t>1 In hand</t>
+        </is>
+      </c>
+      <c r="I5" s="147" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="J5" s="144" t="inlineStr">
+        <is>
+          <t>Planning + FWC/USFWS</t>
+        </is>
+      </c>
+      <c r="K5" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L5" s="144" t="inlineStr">
+        <is>
+          <t>Confirm no listed-species habitat; document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B6" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C6" s="144" t="inlineStr">
+        <is>
+          <t>Wetland &amp; Water Body Conservation</t>
+        </is>
+      </c>
+      <c r="D6" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E6" s="143" t="inlineStr"/>
+      <c r="F6" s="143" t="inlineStr"/>
+      <c r="G6" s="148" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="H6" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I6" s="147" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="J6" s="144" t="inlineStr">
+        <is>
+          <t>Environmental Svcs</t>
+        </is>
+      </c>
+      <c r="K6" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L6" s="144" t="inlineStr">
+        <is>
+          <t>Living shorelines / canal buffers; document seawall condition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B7" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C7" s="144" t="inlineStr">
+        <is>
+          <t>Agricultural Land Conservation</t>
+        </is>
+      </c>
+      <c r="D7" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E7" s="143" t="inlineStr"/>
+      <c r="F7" s="143" t="inlineStr"/>
+      <c r="G7" s="145" t="inlineStr">
+        <is>
+          <t>Met (N/A)</t>
+        </is>
+      </c>
+      <c r="H7" s="150" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I7" s="147" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J7" s="144" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K7" s="143" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L7" s="144" t="inlineStr">
+        <is>
+          <t>No farmland - no action.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B8" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C8" s="144" t="inlineStr">
+        <is>
+          <t>Floodplain Avoidance</t>
+        </is>
+      </c>
+      <c r="D8" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E8" s="143" t="inlineStr"/>
+      <c r="F8" s="143" t="inlineStr"/>
+      <c r="G8" s="148" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="H8" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I8" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J8" s="144" t="inlineStr">
+        <is>
+          <t>Engineering + City</t>
+        </is>
+      </c>
+      <c r="K8" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L8" s="144" t="inlineStr">
+        <is>
+          <t>Qualify via previously-developed path; freeboard + resilient standards (Zone AE); build on FEMA CRS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B9" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C9" s="144" t="inlineStr">
+        <is>
+          <t>Preferred Locations</t>
+        </is>
+      </c>
+      <c r="D9" s="143" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" s="143" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" s="143" t="n">
+        <v>7</v>
+      </c>
+      <c r="G9" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H9" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I9" s="147" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="J9" s="144" t="inlineStr">
+        <is>
+          <t>Planning + consultant</t>
+        </is>
+      </c>
+      <c r="K9" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L9" s="144" t="inlineStr">
+        <is>
+          <t>Commission connectivity/adjacency analysis to claim it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B10" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C10" s="144" t="inlineStr">
+        <is>
+          <t>Brownfield Remediation</t>
+        </is>
+      </c>
+      <c r="D10" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="151" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H10" s="150" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I10" s="147" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J10" s="144" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K10" s="143" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L10" s="144" t="inlineStr">
+        <is>
+          <t>No known brownfield.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B11" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C11" s="144" t="inlineStr">
+        <is>
+          <t>Access to Quality Transit</t>
+        </is>
+      </c>
+      <c r="D11" s="143" t="n">
+        <v>7</v>
+      </c>
+      <c r="E11" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="143" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H11" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I11" s="147" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="J11" s="144" t="inlineStr">
+        <is>
+          <t>BCT + City</t>
+        </is>
+      </c>
+      <c r="K11" s="143" t="inlineStr">
+        <is>
+          <t>$$$</t>
+        </is>
+      </c>
+      <c r="L11" s="144" t="inlineStr">
+        <is>
+          <t>Advocate higher BCT frequency; upgrade shelters; document service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B12" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C12" s="144" t="inlineStr">
+        <is>
+          <t>Bicycle Facilities</t>
+        </is>
+      </c>
+      <c r="D12" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H12" s="152" t="inlineStr">
+        <is>
+          <t>2 City program</t>
+        </is>
+      </c>
+      <c r="I12" s="147" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="J12" s="144" t="inlineStr">
+        <is>
+          <t>City + Broward MPO</t>
+        </is>
+      </c>
+      <c r="K12" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L12" s="144" t="inlineStr">
+        <is>
+          <t>Bike lanes/racks linking Cove node, beach, A1A; join county network.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B13" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C13" s="144" t="inlineStr">
+        <is>
+          <t>Housing &amp; Jobs Proximity</t>
+        </is>
+      </c>
+      <c r="D13" s="143" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H13" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I13" s="147" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="J13" s="144" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="K13" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L13" s="144" t="inlineStr">
+        <is>
+          <t>Document jobs within 1/2 mile (retail + Hillsboro corridor).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B14" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C14" s="144" t="inlineStr">
+        <is>
+          <t>Steep Slope Protection</t>
+        </is>
+      </c>
+      <c r="D14" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="151" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H14" s="150" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I14" s="147" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J14" s="144" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K14" s="143" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L14" s="144" t="inlineStr">
+        <is>
+          <t>Flat coastal site - not achievable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B15" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C15" s="144" t="inlineStr">
+        <is>
+          <t>Site Design for Habitat/Water Body</t>
+        </is>
+      </c>
+      <c r="D15" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="153" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="H15" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I15" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J15" s="144" t="inlineStr">
+        <is>
+          <t>Environmental Svcs</t>
+        </is>
+      </c>
+      <c r="K15" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L15" s="144" t="inlineStr">
+        <is>
+          <t>Native shoreline planting/habitat features to pursue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B16" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C16" s="144" t="inlineStr">
+        <is>
+          <t>Restoration of Habitat/Wetlands</t>
+        </is>
+      </c>
+      <c r="D16" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="153" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="H16" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I16" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J16" s="144" t="inlineStr">
+        <is>
+          <t>Environmental Svcs</t>
+        </is>
+      </c>
+      <c r="K16" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L16" s="144" t="inlineStr">
+        <is>
+          <t>Restore mangrove/native edge (e.g., near Sullivan Park).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="143" t="inlineStr">
+        <is>
+          <t>SLL</t>
+        </is>
+      </c>
+      <c r="B17" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C17" s="144" t="inlineStr">
+        <is>
+          <t>Long-Term Conservation Management</t>
+        </is>
+      </c>
+      <c r="D17" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="153" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="H17" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I17" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J17" s="144" t="inlineStr">
+        <is>
+          <t>Environmental Svcs</t>
+        </is>
+      </c>
+      <c r="K17" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L17" s="144" t="inlineStr">
+        <is>
+          <t>Management plan for any restored habitat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B18" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C18" s="144" t="inlineStr">
+        <is>
+          <t>Walkable Streets</t>
+        </is>
+      </c>
+      <c r="D18" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E18" s="143" t="inlineStr"/>
+      <c r="F18" s="143" t="inlineStr"/>
+      <c r="G18" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H18" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I18" s="147" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="J18" s="144" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="K18" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L18" s="144" t="inlineStr">
+        <is>
+          <t>Sidewalk audit; fill gaps; entries face the street on corridors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B19" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C19" s="144" t="inlineStr">
+        <is>
+          <t>Compact Development</t>
+        </is>
+      </c>
+      <c r="D19" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E19" s="143" t="inlineStr"/>
+      <c r="F19" s="143" t="inlineStr"/>
+      <c r="G19" s="148" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="H19" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I19" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J19" s="144" t="inlineStr">
+        <is>
+          <t>Planning/CRA/Commission</t>
+        </is>
+      </c>
+      <c r="K19" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L19" s="144" t="inlineStr">
+        <is>
+          <t>Raise allowed net density on US-1 &amp; Hillsboro edges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B20" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C20" s="144" t="inlineStr">
+        <is>
+          <t>Connected &amp; Open Community</t>
+        </is>
+      </c>
+      <c r="D20" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E20" s="143" t="inlineStr"/>
+      <c r="F20" s="143" t="inlineStr"/>
+      <c r="G20" s="148" t="inlineStr">
+        <is>
+          <t>At risk</t>
+        </is>
+      </c>
+      <c r="H20" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I20" s="147" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="J20" s="144" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="K20" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L20" s="144" t="inlineStr">
+        <is>
+          <t>Ped cut-throughs; keep streets public &amp; through-connected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B21" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C21" s="144" t="inlineStr">
+        <is>
+          <t>Walkable Streets</t>
+        </is>
+      </c>
+      <c r="D21" s="143" t="n">
+        <v>9</v>
+      </c>
+      <c r="E21" s="143" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" s="143" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H21" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I21" s="147" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="J21" s="144" t="inlineStr">
+        <is>
+          <t>Public Works</t>
+        </is>
+      </c>
+      <c r="K21" s="143" t="inlineStr">
+        <is>
+          <t>$$$</t>
+        </is>
+      </c>
+      <c r="L21" s="144" t="inlineStr">
+        <is>
+          <t>Sidewalks, crossings, calming, street trees on grid + corridors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B22" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C22" s="144" t="inlineStr">
+        <is>
+          <t>Compact Development</t>
+        </is>
+      </c>
+      <c r="D22" s="143" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="153" t="inlineStr">
+        <is>
+          <t>Needs redevelopment</t>
+        </is>
+      </c>
+      <c r="H22" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I22" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J22" s="144" t="inlineStr">
+        <is>
+          <t>Planning/CRA</t>
+        </is>
+      </c>
+      <c r="K22" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L22" s="144" t="inlineStr">
+        <is>
+          <t>Up to 6 with edge rezoning / multifamily infill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B23" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C23" s="144" t="inlineStr">
+        <is>
+          <t>Mixed-Use Neighborhoods</t>
+        </is>
+      </c>
+      <c r="D23" s="143" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H23" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I23" s="147" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="J23" s="144" t="inlineStr">
+        <is>
+          <t>Planning/CRA</t>
+        </is>
+      </c>
+      <c r="K23" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L23" s="144" t="inlineStr">
+        <is>
+          <t>Ground-floor retail + housing at node; more with corridor rezoning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B24" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C24" s="144" t="inlineStr">
+        <is>
+          <t>Housing Types &amp; Affordability</t>
+        </is>
+      </c>
+      <c r="D24" s="143" t="n">
+        <v>7</v>
+      </c>
+      <c r="E24" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="153" t="inlineStr">
+        <is>
+          <t>Needs redevelopment</t>
+        </is>
+      </c>
+      <c r="H24" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I24" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J24" s="144" t="inlineStr">
+        <is>
+          <t>Planning/CRA/Commission</t>
+        </is>
+      </c>
+      <c r="K24" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L24" s="144" t="inlineStr">
+        <is>
+          <t>Up to 7 with diverse + income-restricted corridor housing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B25" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C25" s="144" t="inlineStr">
+        <is>
+          <t>Reduced Parking Footprint</t>
+        </is>
+      </c>
+      <c r="D25" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="153" t="inlineStr">
+        <is>
+          <t>Needs redevelopment</t>
+        </is>
+      </c>
+      <c r="H25" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I25" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J25" s="144" t="inlineStr">
+        <is>
+          <t>CRA</t>
+        </is>
+      </c>
+      <c r="K25" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L25" s="144" t="inlineStr">
+        <is>
+          <t>Shared/structured parking at the shopping center.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B26" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C26" s="144" t="inlineStr">
+        <is>
+          <t>Connected &amp; Open Community</t>
+        </is>
+      </c>
+      <c r="D26" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H26" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I26" s="147" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="J26" s="144" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="K26" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L26" s="144" t="inlineStr">
+        <is>
+          <t>Ped/bike connections; public through-streets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B27" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C27" s="144" t="inlineStr">
+        <is>
+          <t>Transit Facilities</t>
+        </is>
+      </c>
+      <c r="D27" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="145" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="H27" s="146" t="inlineStr">
+        <is>
+          <t>1 In hand</t>
+        </is>
+      </c>
+      <c r="I27" s="147" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="J27" s="144" t="inlineStr">
+        <is>
+          <t>City + BCT</t>
+        </is>
+      </c>
+      <c r="K27" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L27" s="144" t="inlineStr">
+        <is>
+          <t>Maintain shelters/benches; add real-time info.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B28" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C28" s="144" t="inlineStr">
+        <is>
+          <t>Transportation Demand Management</t>
+        </is>
+      </c>
+      <c r="D28" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="153" t="inlineStr">
+        <is>
+          <t>Needs redevelopment</t>
+        </is>
+      </c>
+      <c r="H28" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I28" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J28" s="144" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="K28" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L28" s="144" t="inlineStr">
+        <is>
+          <t>TDM program tied to redevelopment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B29" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C29" s="144" t="inlineStr">
+        <is>
+          <t>Access to Civic &amp; Public Space</t>
+        </is>
+      </c>
+      <c r="D29" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="145" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="H29" s="146" t="inlineStr">
+        <is>
+          <t>1 In hand</t>
+        </is>
+      </c>
+      <c r="I29" s="147" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="J29" s="144" t="inlineStr">
+        <is>
+          <t>Planning/Parks</t>
+        </is>
+      </c>
+      <c r="K29" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L29" s="144" t="inlineStr">
+        <is>
+          <t>Document Sullivan Park promenade / public waterfront.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B30" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C30" s="144" t="inlineStr">
+        <is>
+          <t>Access to Recreation Facilities</t>
+        </is>
+      </c>
+      <c r="D30" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="145" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="H30" s="146" t="inlineStr">
+        <is>
+          <t>1 In hand</t>
+        </is>
+      </c>
+      <c r="I30" s="147" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="J30" s="144" t="inlineStr">
+        <is>
+          <t>Parks</t>
+        </is>
+      </c>
+      <c r="K30" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L30" s="144" t="inlineStr">
+        <is>
+          <t>Document parks, pier, beach, Deerfield Island access.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B31" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C31" s="144" t="inlineStr">
+        <is>
+          <t>Visitability &amp; Universal Design</t>
+        </is>
+      </c>
+      <c r="D31" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="153" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="H31" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I31" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J31" s="144" t="inlineStr">
+        <is>
+          <t>Building Dept.</t>
+        </is>
+      </c>
+      <c r="K31" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L31" s="144" t="inlineStr">
+        <is>
+          <t>Adopt visitability standards for new/renovated homes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B32" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C32" s="144" t="inlineStr">
+        <is>
+          <t>Community Outreach &amp; Involvement</t>
+        </is>
+      </c>
+      <c r="D32" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="G32" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H32" s="146" t="inlineStr">
+        <is>
+          <t>1 In hand</t>
+        </is>
+      </c>
+      <c r="I32" s="147" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="J32" s="144" t="inlineStr">
+        <is>
+          <t>Cove Civic Assoc. + Planning</t>
+        </is>
+      </c>
+      <c r="K32" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L32" s="144" t="inlineStr">
+        <is>
+          <t>Formalize charrette/engagement process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B33" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C33" s="144" t="inlineStr">
+        <is>
+          <t>Local Food Production</t>
+        </is>
+      </c>
+      <c r="D33" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="145" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="H33" s="146" t="inlineStr">
+        <is>
+          <t>1 In hand</t>
+        </is>
+      </c>
+      <c r="I33" s="147" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="J33" s="144" t="inlineStr">
+        <is>
+          <t>Cove Civic Assoc.</t>
+        </is>
+      </c>
+      <c r="K33" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L33" s="144" t="inlineStr">
+        <is>
+          <t>Sustain the farmers market; add community garden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B34" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C34" s="144" t="inlineStr">
+        <is>
+          <t>Tree-Lined &amp; Shaded Streetscapes</t>
+        </is>
+      </c>
+      <c r="D34" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H34" s="152" t="inlineStr">
+        <is>
+          <t>2 City program</t>
+        </is>
+      </c>
+      <c r="I34" s="147" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="J34" s="144" t="inlineStr">
+        <is>
+          <t>Environmental Svcs</t>
+        </is>
+      </c>
+      <c r="K34" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L34" s="144" t="inlineStr">
+        <is>
+          <t>Deploy Shady Street Tree program + giveaways; canopy inventory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="143" t="inlineStr">
+        <is>
+          <t>NPD</t>
+        </is>
+      </c>
+      <c r="B35" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C35" s="144" t="inlineStr">
+        <is>
+          <t>Neighborhood Schools</t>
+        </is>
+      </c>
+      <c r="D35" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="145" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="H35" s="146" t="inlineStr">
+        <is>
+          <t>1 In hand</t>
+        </is>
+      </c>
+      <c r="I35" s="147" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="J35" s="144" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="K35" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L35" s="144" t="inlineStr">
+        <is>
+          <t>Document walk access to St. Ambrose / Deerfield schools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B36" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C36" s="144" t="inlineStr">
+        <is>
+          <t>Certified Green Building</t>
+        </is>
+      </c>
+      <c r="D36" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E36" s="143" t="inlineStr"/>
+      <c r="F36" s="143" t="inlineStr"/>
+      <c r="G36" s="153" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="H36" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I36" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J36" s="144" t="inlineStr">
+        <is>
+          <t>Commission/Building</t>
+        </is>
+      </c>
+      <c r="K36" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L36" s="144" t="inlineStr">
+        <is>
+          <t>Require &gt;=1 green-certified building on new construction/major reno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B37" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C37" s="144" t="inlineStr">
+        <is>
+          <t>Minimum Building Energy Performance</t>
+        </is>
+      </c>
+      <c r="D37" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E37" s="143" t="inlineStr"/>
+      <c r="F37" s="143" t="inlineStr"/>
+      <c r="G37" s="153" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="H37" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I37" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J37" s="144" t="inlineStr">
+        <is>
+          <t>Building Dept.</t>
+        </is>
+      </c>
+      <c r="K37" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L37" s="144" t="inlineStr">
+        <is>
+          <t>Energy-code compliance + retrofit incentives; document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B38" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C38" s="144" t="inlineStr">
+        <is>
+          <t>Indoor Water Use Reduction</t>
+        </is>
+      </c>
+      <c r="D38" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E38" s="143" t="inlineStr"/>
+      <c r="F38" s="143" t="inlineStr"/>
+      <c r="G38" s="148" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H38" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I38" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J38" s="144" t="inlineStr">
+        <is>
+          <t>Building Dept.</t>
+        </is>
+      </c>
+      <c r="K38" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L38" s="144" t="inlineStr">
+        <is>
+          <t>Low-flow fixture standards; document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B39" s="143" t="inlineStr">
+        <is>
+          <t>Prereq</t>
+        </is>
+      </c>
+      <c r="C39" s="144" t="inlineStr">
+        <is>
+          <t>Construction Activity Pollution Prevention</t>
+        </is>
+      </c>
+      <c r="D39" s="143" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="E39" s="143" t="inlineStr"/>
+      <c r="F39" s="143" t="inlineStr"/>
+      <c r="G39" s="151" t="inlineStr">
+        <is>
+          <t>N/A now</t>
+        </is>
+      </c>
+      <c r="H39" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I39" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J39" s="144" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="K39" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L39" s="144" t="inlineStr">
+        <is>
+          <t>SWPPP/erosion control on future projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B40" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C40" s="144" t="inlineStr">
+        <is>
+          <t>Certified Green Buildings</t>
+        </is>
+      </c>
+      <c r="D40" s="143" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="153" t="inlineStr">
+        <is>
+          <t>Needs redevelopment</t>
+        </is>
+      </c>
+      <c r="H40" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I40" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J40" s="144" t="inlineStr">
+        <is>
+          <t>Commission/Building</t>
+        </is>
+      </c>
+      <c r="K40" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L40" s="144" t="inlineStr">
+        <is>
+          <t>Incentivize/require green certification for redevelopment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B41" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C41" s="144" t="inlineStr">
+        <is>
+          <t>Optimize Building Energy Performance</t>
+        </is>
+      </c>
+      <c r="D41" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="153" t="inlineStr">
+        <is>
+          <t>Needs redevelopment</t>
+        </is>
+      </c>
+      <c r="H41" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I41" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J41" s="144" t="inlineStr">
+        <is>
+          <t>Building Dept.</t>
+        </is>
+      </c>
+      <c r="K41" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L41" s="144" t="inlineStr">
+        <is>
+          <t>Efficiency retrofits; high-performance envelope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B42" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C42" s="144" t="inlineStr">
+        <is>
+          <t>Indoor Water Use Reduction</t>
+        </is>
+      </c>
+      <c r="D42" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="153" t="inlineStr">
+        <is>
+          <t>Needs redevelopment</t>
+        </is>
+      </c>
+      <c r="H42" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I42" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J42" s="144" t="inlineStr">
+        <is>
+          <t>Building Dept.</t>
+        </is>
+      </c>
+      <c r="K42" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L42" s="144" t="inlineStr">
+        <is>
+          <t>Low-flow retrofit program.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B43" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C43" s="144" t="inlineStr">
+        <is>
+          <t>Outdoor Water Use Reduction</t>
+        </is>
+      </c>
+      <c r="D43" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H43" s="152" t="inlineStr">
+        <is>
+          <t>2 City program</t>
+        </is>
+      </c>
+      <c r="I43" s="147" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="J43" s="144" t="inlineStr">
+        <is>
+          <t>Cove Civic Assoc. + UF/IFAS</t>
+        </is>
+      </c>
+      <c r="K43" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L43" s="144" t="inlineStr">
+        <is>
+          <t>Enroll in Broward NatureScape / Florida-Friendly Landscaping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B44" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C44" s="144" t="inlineStr">
+        <is>
+          <t>Building Reuse</t>
+        </is>
+      </c>
+      <c r="D44" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="145" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="H44" s="146" t="inlineStr">
+        <is>
+          <t>1 In hand</t>
+        </is>
+      </c>
+      <c r="I44" s="147" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="J44" s="144" t="inlineStr">
+        <is>
+          <t>Planning/Building</t>
+        </is>
+      </c>
+      <c r="K44" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L44" s="144" t="inlineStr">
+        <is>
+          <t>Reuse-over-teardown preference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B45" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C45" s="144" t="inlineStr">
+        <is>
+          <t>Historic Resource Preservation / Adaptive Reuse</t>
+        </is>
+      </c>
+      <c r="D45" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H45" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I45" s="147" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="J45" s="144" t="inlineStr">
+        <is>
+          <t>Planning + Historical Society</t>
+        </is>
+      </c>
+      <c r="K45" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L45" s="144" t="inlineStr">
+        <is>
+          <t>Leverage Butler House; consider local designation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B46" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C46" s="144" t="inlineStr">
+        <is>
+          <t>Minimized Site Disturbance</t>
+        </is>
+      </c>
+      <c r="D46" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="151" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H46" s="150" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I46" s="147" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J46" s="144" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K46" s="143" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L46" s="144" t="inlineStr">
+        <is>
+          <t>Built-out; applies to infill only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B47" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C47" s="144" t="inlineStr">
+        <is>
+          <t>Rainwater Management</t>
+        </is>
+      </c>
+      <c r="D47" s="143" t="n">
+        <v>4</v>
+      </c>
+      <c r="E47" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H47" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I47" s="147" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="J47" s="144" t="inlineStr">
+        <is>
+          <t>Engineering/Stormwater</t>
+        </is>
+      </c>
+      <c r="K47" s="143" t="inlineStr">
+        <is>
+          <t>$$$</t>
+        </is>
+      </c>
+      <c r="L47" s="144" t="inlineStr">
+        <is>
+          <t>Green stormwater at retail lot &amp; ROW; leverage FEMA CRS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B48" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C48" s="144" t="inlineStr">
+        <is>
+          <t>Heat Island Reduction</t>
+        </is>
+      </c>
+      <c r="D48" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H48" s="152" t="inlineStr">
+        <is>
+          <t>2 City program</t>
+        </is>
+      </c>
+      <c r="I48" s="147" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="J48" s="144" t="inlineStr">
+        <is>
+          <t>Environmental Svcs</t>
+        </is>
+      </c>
+      <c r="K48" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L48" s="144" t="inlineStr">
+        <is>
+          <t>Shade trees + cool/permeable surfaces at the lot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B49" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C49" s="144" t="inlineStr">
+        <is>
+          <t>Solar Orientation</t>
+        </is>
+      </c>
+      <c r="D49" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="151" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H49" s="150" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I49" s="147" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J49" s="144" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K49" s="143" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L49" s="144" t="inlineStr">
+        <is>
+          <t>Applies to new layout only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B50" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C50" s="144" t="inlineStr">
+        <is>
+          <t>Renewable Energy Production</t>
+        </is>
+      </c>
+      <c r="D50" s="143" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="153" t="inlineStr">
+        <is>
+          <t>Needs redevelopment</t>
+        </is>
+      </c>
+      <c r="H50" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I50" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J50" s="144" t="inlineStr">
+        <is>
+          <t>Building/residents</t>
+        </is>
+      </c>
+      <c r="K50" s="143" t="inlineStr">
+        <is>
+          <t>$$$</t>
+        </is>
+      </c>
+      <c r="L50" s="144" t="inlineStr">
+        <is>
+          <t>Rooftop/community solar program.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B51" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C51" s="144" t="inlineStr">
+        <is>
+          <t>District Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="D51" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E51" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="151" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H51" s="150" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I51" s="147" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J51" s="144" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K51" s="143" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L51" s="144" t="inlineStr">
+        <is>
+          <t>Not viable at this scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B52" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C52" s="144" t="inlineStr">
+        <is>
+          <t>Infrastructure Energy Efficiency</t>
+        </is>
+      </c>
+      <c r="D52" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H52" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I52" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J52" s="144" t="inlineStr">
+        <is>
+          <t>Public Works</t>
+        </is>
+      </c>
+      <c r="K52" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L52" s="144" t="inlineStr">
+        <is>
+          <t>LED streetlights; efficient stormwater pumps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B53" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C53" s="144" t="inlineStr">
+        <is>
+          <t>Wastewater Management</t>
+        </is>
+      </c>
+      <c r="D53" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="148" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="H53" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I53" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J53" s="144" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="K53" s="143" t="inlineStr">
+        <is>
+          <t>$$$</t>
+        </is>
+      </c>
+      <c r="L53" s="144" t="inlineStr">
+        <is>
+          <t>Greywater/reuse; nutrient reduction to protect ICW.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B54" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C54" s="144" t="inlineStr">
+        <is>
+          <t>Recycled and Reused Infrastructure</t>
+        </is>
+      </c>
+      <c r="D54" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="153" t="inlineStr">
+        <is>
+          <t>Not met</t>
+        </is>
+      </c>
+      <c r="H54" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I54" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J54" s="144" t="inlineStr">
+        <is>
+          <t>Public Works</t>
+        </is>
+      </c>
+      <c r="K54" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L54" s="144" t="inlineStr">
+        <is>
+          <t>Reuse road base/materials in ROW projects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B55" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C55" s="144" t="inlineStr">
+        <is>
+          <t>Solid Waste Management</t>
+        </is>
+      </c>
+      <c r="D55" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E55" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="145" t="inlineStr">
+        <is>
+          <t>Met</t>
+        </is>
+      </c>
+      <c r="H55" s="146" t="inlineStr">
+        <is>
+          <t>1 In hand</t>
+        </is>
+      </c>
+      <c r="I55" s="147" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="J55" s="144" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="K55" s="143" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="L55" s="144" t="inlineStr">
+        <is>
+          <t>Maintain recycling; add construction-waste diversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="143" t="inlineStr">
+        <is>
+          <t>GIB</t>
+        </is>
+      </c>
+      <c r="B56" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C56" s="144" t="inlineStr">
+        <is>
+          <t>Light Pollution Reduction</t>
+        </is>
+      </c>
+      <c r="D56" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H56" s="146" t="inlineStr">
+        <is>
+          <t>1 In hand</t>
+        </is>
+      </c>
+      <c r="I56" s="147" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="J56" s="144" t="inlineStr">
+        <is>
+          <t>Public Works/Code</t>
+        </is>
+      </c>
+      <c r="K56" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L56" s="144" t="inlineStr">
+        <is>
+          <t>Extend sea-turtle/dark-sky lighting standard inland.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="143" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B57" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C57" s="144" t="inlineStr">
+        <is>
+          <t>Innovation</t>
+        </is>
+      </c>
+      <c r="D57" s="143" t="n">
+        <v>5</v>
+      </c>
+      <c r="E57" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="153" t="inlineStr">
+        <is>
+          <t>Needs redevelopment</t>
+        </is>
+      </c>
+      <c r="H57" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I57" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J57" s="144" t="inlineStr">
+        <is>
+          <t>Project team</t>
+        </is>
+      </c>
+      <c r="K57" s="143" t="inlineStr">
+        <is>
+          <t>policy</t>
+        </is>
+      </c>
+      <c r="L57" s="144" t="inlineStr">
+        <is>
+          <t>Pilot exemplary strategies (resilience / living shoreline).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="143" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B58" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C58" s="144" t="inlineStr">
+        <is>
+          <t>LEED Accredited Professional</t>
+        </is>
+      </c>
+      <c r="D58" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="153" t="inlineStr">
+        <is>
+          <t>Needs redevelopment</t>
+        </is>
+      </c>
+      <c r="H58" s="154" t="inlineStr">
+        <is>
+          <t>4 Redevelopment</t>
+        </is>
+      </c>
+      <c r="I58" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J58" s="144" t="inlineStr">
+        <is>
+          <t>Project team</t>
+        </is>
+      </c>
+      <c r="K58" s="143" t="inlineStr">
+        <is>
+          <t>$$</t>
+        </is>
+      </c>
+      <c r="L58" s="144" t="inlineStr">
+        <is>
+          <t>Engage a LEED AP on any redevelopment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="143" t="inlineStr">
+        <is>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="B59" s="143" t="inlineStr">
+        <is>
+          <t>Credit</t>
+        </is>
+      </c>
+      <c r="C59" s="144" t="inlineStr">
+        <is>
+          <t>Regional Priority (x4, Region Defined)</t>
+        </is>
+      </c>
+      <c r="D59" s="143" t="n">
+        <v>4</v>
+      </c>
+      <c r="E59" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="148" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="H59" s="149" t="inlineStr">
+        <is>
+          <t>3 Capital/analysis</t>
+        </is>
+      </c>
+      <c r="I59" s="147" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="J59" s="144" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="K59" s="143" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L59" s="144" t="inlineStr">
+        <is>
+          <t>Pursue FL RP credits (rainwater/heat/water) once underlying earned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="C61" s="155" t="inlineStr">
+        <is>
+          <t>SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="C62" s="156" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D62" s="156" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="E62" s="156" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="F62" s="156" t="inlineStr">
+        <is>
+          <t>Achiev.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="C63" s="157" t="inlineStr">
+        <is>
+          <t>Smart Location &amp; Linkage</t>
+        </is>
+      </c>
+      <c r="D63" s="143" t="n">
+        <v>28</v>
+      </c>
+      <c r="E63" s="143" t="n">
+        <v>7</v>
+      </c>
+      <c r="F63" s="143" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="C64" s="157" t="inlineStr">
+        <is>
+          <t>Neighborhood Pattern &amp; Design</t>
+        </is>
+      </c>
+      <c r="D64" s="143" t="n">
+        <v>41</v>
+      </c>
+      <c r="E64" s="143" t="n">
+        <v>11</v>
+      </c>
+      <c r="F64" s="143" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="C65" s="157" t="inlineStr">
+        <is>
+          <t>Green Infrastructure &amp; Buildings</t>
+        </is>
+      </c>
+      <c r="D65" s="143" t="n">
+        <v>31</v>
+      </c>
+      <c r="E65" s="143" t="n">
+        <v>2</v>
+      </c>
+      <c r="F65" s="143" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="C66" s="157" t="inlineStr">
+        <is>
+          <t>Innovation &amp; Design Process</t>
+        </is>
+      </c>
+      <c r="D66" s="143" t="n">
+        <v>6</v>
+      </c>
+      <c r="E66" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" s="143" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="C67" s="157" t="inlineStr">
+        <is>
+          <t>Regional Priority</t>
+        </is>
+      </c>
+      <c r="D67" s="143" t="n">
+        <v>4</v>
+      </c>
+      <c r="E67" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="143" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="C68" s="158" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D68" s="159" t="n">
+        <v>110</v>
+      </c>
+      <c r="E68" s="159" t="n">
+        <v>20</v>
+      </c>
+      <c r="F68" s="159" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="C70" s="140" t="inlineStr">
+        <is>
+          <t>Now (as-is): ~20 pts  |  Achievable without rezoning (Tiers 1-3): ~39 pts  |  Max: 110  |  Certified 40-49 / Silver 50-59 / Gold 60-79 / Platinum 80+.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="C71" s="140" t="inlineStr">
+        <is>
+          <t>The ~39-pt 'Achievable' column is the improvement ceiling with NO rezoning/new buildings; the Action Plan tab sequences ~33 of it across Year 1-3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="C72" s="140" t="inlineStr">
+        <is>
+          <t>Tier 4 (red) = only reachable through redevelopment / rezoning the US-1 &amp; Hillsboro edges + a green-building requirement - the path from ~39 toward Certified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="C73" s="140" t="inlineStr">
+        <is>
+          <t>LEED-ND rates NEW development; this is an interpretive read of an existing district for planning use. Boundary = official Cove Waterfront District study area (KMZ).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:L59"/>
+  <mergeCells count="6">
+    <mergeCell ref="C71:L71"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="C70:L70"/>
+    <mergeCell ref="C73:L73"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="C72:L72"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1293,6 +4758,11 @@
           <t>YEAR 1  -  DOCUMENT &amp; QUICK WINS  (mostly free; claim what's already true)</t>
         </is>
       </c>
+      <c r="B5" s="138" t="n"/>
+      <c r="C5" s="138" t="n"/>
+      <c r="D5" s="138" t="n"/>
+      <c r="E5" s="138" t="n"/>
+      <c r="F5" s="139" t="n"/>
     </row>
     <row r="6" ht="44" customHeight="1">
       <c r="A6" s="121" t="inlineStr">
@@ -1498,6 +4968,11 @@
           <t>YEAR 2  -  PROGRAMS MATURE + FIRST ANALYSES  (low-moderate cost)</t>
         </is>
       </c>
+      <c r="B14" s="138" t="n"/>
+      <c r="C14" s="138" t="n"/>
+      <c r="D14" s="138" t="n"/>
+      <c r="E14" s="138" t="n"/>
+      <c r="F14" s="139" t="n"/>
     </row>
     <row r="15" ht="44" customHeight="1">
       <c r="A15" s="125" t="inlineStr">
@@ -1703,6 +5178,11 @@
           <t>YEAR 3  -  CAPITAL PROJECTS &amp; GREEN INFRASTRUCTURE  (budget required; still NO rezoning)</t>
         </is>
       </c>
+      <c r="B23" s="138" t="n"/>
+      <c r="C23" s="138" t="n"/>
+      <c r="D23" s="138" t="n"/>
+      <c r="E23" s="138" t="n"/>
+      <c r="F23" s="139" t="n"/>
     </row>
     <row r="24" ht="44" customHeight="1">
       <c r="A24" s="129" t="inlineStr">
@@ -1848,6 +5328,11 @@
           <t>ONGOING / FUTURE  -  TIER 4 POLICY TRACK  (not counted below - this is the path PAST ~33 toward Certified)</t>
         </is>
       </c>
+      <c r="B30" s="138" t="n"/>
+      <c r="C30" s="138" t="n"/>
+      <c r="D30" s="138" t="n"/>
+      <c r="E30" s="138" t="n"/>
+      <c r="F30" s="139" t="n"/>
     </row>
     <row r="31" ht="44" customHeight="1">
       <c r="A31" s="133" t="inlineStr">
@@ -1919,6 +5404,11 @@
           <t>TOTAL INTEGRATED WITH NO REZONING / NO NEW BUILDINGS:  ~33 LEED-ND points over 3 years</t>
         </is>
       </c>
+      <c r="B34" s="138" t="n"/>
+      <c r="C34" s="138" t="n"/>
+      <c r="D34" s="138" t="n"/>
+      <c r="E34" s="138" t="n"/>
+      <c r="F34" s="139" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="119" t="inlineStr">
@@ -1966,7 +5456,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2611,7 +6101,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4603,7 +8093,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6880,7 +10370,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Ground the plan in the Sustainable Neighborhoods manual (code/policy amendments)
Incorporate the Technical Guidance Manual for Sustainable Neighborhoods
(Global Green/EPA) the user supplied: add a 'Local plan/code/policy to amend'
column to the Action Plan sheet, mapping each of the 10 actions to the specific
instrument to amend (comprehensive plan, zoning, subdivision & site-plan regs,
capital improvement program, lighting/landscape ordinances) using the manual's
own strategies. Add a method note + LEED-ND 2009-vs-v4 version caveat.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C83XSMHt5roS8jvvJWFf8j
</commit_message>
<xml_diff>
--- a/the_cove_deerfield_beach/the_cove_LEED_ND_scorecard.xlsx
+++ b/the_cove_deerfield_beach/the_cove_LEED_ND_scorecard.xlsx
@@ -214,7 +214,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -282,8 +282,13 @@
         <fgColor rgb="00F5EADC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F0E7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -422,11 +427,55 @@
         <color rgb="00D0D0D0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D0D0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -812,6 +861,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="12" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1114,32 +1169,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="102" t="inlineStr">
         <is>
-          <t>The Cove - Improvement Plan (the actions behind the score)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
+          <t>The Cove - Improvement Plan: using LEED-ND to amend local plans, codes &amp; policies</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
       <c r="A2" s="103" t="inlineStr">
         <is>
-          <t>Today ~20 pts  -&gt;  after this plan ~35 pts (no rezoning)  -&gt;  LEED Certified 40 (needs Phase 3).  Points are rough direction; see the scored rubric on the 'Neighborhood Development' sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
+          <t>Method follows the Technical Guidance Manual for Sustainable Neighborhoods (Global Green / EPA): evaluate the district against LEED-ND, then amend the local plan/code/policy behind each credit.  Today ~20 pts -&gt; after this plan ~35 (no rezoning) -&gt; Certified 40 (needs Phase 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1">
       <c r="A3" s="104" t="inlineStr">
         <is>
           <t>#</t>
@@ -1168,6 +1224,11 @@
       <c r="F3" s="105" t="inlineStr">
         <is>
           <t>LEED-ND credit(s)</t>
+        </is>
+      </c>
+      <c r="G3" s="121" t="inlineStr">
+        <is>
+          <t>Local plan / code / policy to amend  (per the Sustainable Neighborhoods manual)</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1239,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="46" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="107" t="n">
         <v>1</v>
       </c>
@@ -1199,7 +1260,7 @@
       </c>
       <c r="E5" s="109" t="inlineStr">
         <is>
-          <t>Instantly counts toward the score; makes you grant-ready.</t>
+          <t>Instantly counts toward the score; grant-ready.</t>
         </is>
       </c>
       <c r="F5" s="110" t="inlineStr">
@@ -1207,8 +1268,13 @@
           <t>6 credits: Civic Space, Recreation, Local Food, Schools, Transit Facilities, Solid Waste</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="46" customHeight="1">
+      <c r="G5" s="122" t="inlineStr">
+        <is>
+          <t>Neighborhood / comprehensive plan - baseline 'existing conditions' inventory (the manual's Step 1: evaluate local plans against LEED-ND).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="107" t="n">
         <v>2</v>
       </c>
@@ -1237,8 +1303,13 @@
           <t>Tree-Lined Streetscapes; Heat Island</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="46" customHeight="1">
+      <c r="G6" s="122" t="inlineStr">
+        <is>
+          <t>Subdivision &amp; site-plan regs (street-tree/landscape standards) + Capital Improvement Program - require tree-lined, shaded streets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
       <c r="A7" s="107" t="n">
         <v>3</v>
       </c>
@@ -1267,8 +1338,13 @@
           <t>Outdoor Water Use Reduction</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="46" customHeight="1">
+      <c r="G7" s="122" t="inlineStr">
+        <is>
+          <t>Landscape ordinance / site-plan regs - 'amend site plan &amp; subdivision regulations to require water-efficient landscaping' (manual, GIBc4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
       <c r="A8" s="107" t="n">
         <v>4</v>
       </c>
@@ -1297,8 +1373,13 @@
           <t>Light Pollution Reduction</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="46" customHeight="1">
+      <c r="G8" s="122" t="inlineStr">
+        <is>
+          <t>Outdoor-lighting ordinance / zoning - dark-sky lighting standards (manual, GIBc17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
       <c r="A9" s="107" t="n">
         <v>5</v>
       </c>
@@ -1327,6 +1408,11 @@
           <t>Community Outreach &amp; Involvement</t>
         </is>
       </c>
+      <c r="G9" s="122" t="inlineStr">
+        <is>
+          <t>Development-review procedures - 'amend review procedures to include community-outreach steps' (manual, NPDc12).</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="111" t="inlineStr">
@@ -1335,7 +1421,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="46" customHeight="1">
+    <row r="11" ht="58" customHeight="1">
       <c r="A11" s="112" t="n">
         <v>6</v>
       </c>
@@ -1364,8 +1450,13 @@
           <t>Walkable Streets; Bicycle Facilities</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="46" customHeight="1">
+      <c r="G11" s="122" t="inlineStr">
+        <is>
+          <t>Subdivision &amp; site-plan regs (sidewalk/pavement/connectivity standards) + Capital Improvement Program (build them) - manual NPDp1/c1, SLLc4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
       <c r="A12" s="112" t="n">
         <v>7</v>
       </c>
@@ -1394,8 +1485,13 @@
           <t>Access to Quality Transit</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="46" customHeight="1">
+      <c r="G12" s="122" t="inlineStr">
+        <is>
+          <t>Capital Improvement Program + comp-plan transportation element (coordinate w/ BCT) - transit facilities (manual, NPDc7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
       <c r="A13" s="112" t="n">
         <v>8</v>
       </c>
@@ -1424,8 +1520,13 @@
           <t>Rainwater Management (+ FEMA CRS)</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="46" customHeight="1">
+      <c r="G13" s="122" t="inlineStr">
+        <is>
+          <t>Subdivision &amp; site-plan regs (stormwater / pavement standards) + Capital Improvement Program - green stormwater (manual, GIBc8/GIBc9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="58" customHeight="1">
       <c r="A14" s="112" t="n">
         <v>9</v>
       </c>
@@ -1454,6 +1555,11 @@
           <t>Preferred Locations; Housing &amp; Jobs Proximity</t>
         </is>
       </c>
+      <c r="G14" s="122" t="inlineStr">
+        <is>
+          <t>Neighborhood / comprehensive plan - smart-location &amp; street-network analysis (manual, SLLc1, NPDc6).</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="116" t="inlineStr">
@@ -1462,7 +1568,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="46" customHeight="1">
+    <row r="16" ht="58" customHeight="1">
       <c r="A16" s="117" t="n">
         <v>10</v>
       </c>
@@ -1491,14 +1597,59 @@
           <t>Compact Development; Housing Types; Certified Green Buildings; Energy</t>
         </is>
       </c>
+      <c r="G16" s="122" t="inlineStr">
+        <is>
+          <t>Zoning code (mixed-use/density overlay or form-based code) + comprehensive plan + energy/building code green-building requirement (manual, NPDc2/c4, GIBp1/c1/c2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="103" t="inlineStr">
+        <is>
+          <t>METHOD (per the Technical Guidance Manual for Sustainable Neighborhoods, Global Green USA / U.S. EPA, 2012-13):</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1) Evaluate the district's existing plans, codes &amp; policies against the LEED-ND rating system;  2) Amend the specific instrument behind each credit -</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  comprehensive/neighborhood plan, zoning code, subdivision &amp; site-plan regulations, capital improvement program, and design/lighting/landscape ordinances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="103" t="inlineStr">
+        <is>
+          <t>NOTE ON VERSIONS: the manual cites LEED-ND 2009 credit numbers (e.g., GIBc4, NPDc1); the scored rubric on the 'Neighborhood Development' sheet is LEED v4 for ND.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  The credit intents map across the two versions; only the numbering/labels differ.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A15:F15"/>
+  <mergeCells count="10">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>